<commit_message>
Prepare Unity Assignment v1.0.13 scenarios and NCM selection
Add optional NCM scenarios, claimant-state dropdown resolution, and single-session lookup behavior. Preserve upstream CMS task IDs and record the independently verified release build.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Processes/Unity/Stand-Alone/Unity-Input.xlsx
+++ b/Processes/Unity/Stand-Alone/Unity-Input.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Unity Input'!$A$1:$AI$501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Unity Input'!$A$1:$AJ$501</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -207,7 +207,7 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Leave unknown values blank.</t>
+        <t>Optional. Up to 32,767 characters (Excel-compatible). Line breaks and leading/trailing whitespace are preserved when loaded.</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
@@ -338,6 +338,11 @@
     <comment ref="AI1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Leave unknown values blank.</t>
+      </text>
+    </comment>
+    <comment ref="AJ1" authorId="0" shapeId="0">
+      <text>
+        <t>Exact full NCM name. Required only for Scenario 2 in All/Assign; claimant first and last names are also required in that scenario.</t>
       </text>
     </comment>
   </commentList>
@@ -633,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI501"/>
+  <dimension ref="A1:AJ501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -671,6 +676,7 @@
     <col width="25" customWidth="1" min="33" max="33"/>
     <col width="25" customWidth="1" min="34" max="34"/>
     <col width="25" customWidth="1" min="35" max="35"/>
+    <col width="25" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
@@ -849,6 +855,11 @@
           <t>Attorney - Phone</t>
         </is>
       </c>
+      <c r="AJ1" s="2" t="inlineStr">
+        <is>
+          <t>NCM - NCM full name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -886,6 +897,7 @@
       <c r="AG2" s="3" t="n"/>
       <c r="AH2" s="3" t="n"/>
       <c r="AI2" s="3" t="n"/>
+      <c r="AJ2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -923,6 +935,7 @@
       <c r="AG3" s="3" t="n"/>
       <c r="AH3" s="3" t="n"/>
       <c r="AI3" s="3" t="n"/>
+      <c r="AJ3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -960,6 +973,7 @@
       <c r="AG4" s="3" t="n"/>
       <c r="AH4" s="3" t="n"/>
       <c r="AI4" s="3" t="n"/>
+      <c r="AJ4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -997,6 +1011,7 @@
       <c r="AG5" s="3" t="n"/>
       <c r="AH5" s="3" t="n"/>
       <c r="AI5" s="3" t="n"/>
+      <c r="AJ5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -1034,6 +1049,7 @@
       <c r="AG6" s="3" t="n"/>
       <c r="AH6" s="3" t="n"/>
       <c r="AI6" s="3" t="n"/>
+      <c r="AJ6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -1071,6 +1087,7 @@
       <c r="AG7" s="3" t="n"/>
       <c r="AH7" s="3" t="n"/>
       <c r="AI7" s="3" t="n"/>
+      <c r="AJ7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -1108,6 +1125,7 @@
       <c r="AG8" s="3" t="n"/>
       <c r="AH8" s="3" t="n"/>
       <c r="AI8" s="3" t="n"/>
+      <c r="AJ8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -1145,6 +1163,7 @@
       <c r="AG9" s="3" t="n"/>
       <c r="AH9" s="3" t="n"/>
       <c r="AI9" s="3" t="n"/>
+      <c r="AJ9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -1182,6 +1201,7 @@
       <c r="AG10" s="3" t="n"/>
       <c r="AH10" s="3" t="n"/>
       <c r="AI10" s="3" t="n"/>
+      <c r="AJ10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -1219,6 +1239,7 @@
       <c r="AG11" s="3" t="n"/>
       <c r="AH11" s="3" t="n"/>
       <c r="AI11" s="3" t="n"/>
+      <c r="AJ11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -1256,6 +1277,7 @@
       <c r="AG12" s="3" t="n"/>
       <c r="AH12" s="3" t="n"/>
       <c r="AI12" s="3" t="n"/>
+      <c r="AJ12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -1293,6 +1315,7 @@
       <c r="AG13" s="3" t="n"/>
       <c r="AH13" s="3" t="n"/>
       <c r="AI13" s="3" t="n"/>
+      <c r="AJ13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -1330,6 +1353,7 @@
       <c r="AG14" s="3" t="n"/>
       <c r="AH14" s="3" t="n"/>
       <c r="AI14" s="3" t="n"/>
+      <c r="AJ14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -1367,6 +1391,7 @@
       <c r="AG15" s="3" t="n"/>
       <c r="AH15" s="3" t="n"/>
       <c r="AI15" s="3" t="n"/>
+      <c r="AJ15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -1404,6 +1429,7 @@
       <c r="AG16" s="3" t="n"/>
       <c r="AH16" s="3" t="n"/>
       <c r="AI16" s="3" t="n"/>
+      <c r="AJ16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -1441,6 +1467,7 @@
       <c r="AG17" s="3" t="n"/>
       <c r="AH17" s="3" t="n"/>
       <c r="AI17" s="3" t="n"/>
+      <c r="AJ17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -1478,6 +1505,7 @@
       <c r="AG18" s="3" t="n"/>
       <c r="AH18" s="3" t="n"/>
       <c r="AI18" s="3" t="n"/>
+      <c r="AJ18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -1515,6 +1543,7 @@
       <c r="AG19" s="3" t="n"/>
       <c r="AH19" s="3" t="n"/>
       <c r="AI19" s="3" t="n"/>
+      <c r="AJ19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -1552,6 +1581,7 @@
       <c r="AG20" s="3" t="n"/>
       <c r="AH20" s="3" t="n"/>
       <c r="AI20" s="3" t="n"/>
+      <c r="AJ20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -1589,6 +1619,7 @@
       <c r="AG21" s="3" t="n"/>
       <c r="AH21" s="3" t="n"/>
       <c r="AI21" s="3" t="n"/>
+      <c r="AJ21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -1626,6 +1657,7 @@
       <c r="AG22" s="3" t="n"/>
       <c r="AH22" s="3" t="n"/>
       <c r="AI22" s="3" t="n"/>
+      <c r="AJ22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -1663,6 +1695,7 @@
       <c r="AG23" s="3" t="n"/>
       <c r="AH23" s="3" t="n"/>
       <c r="AI23" s="3" t="n"/>
+      <c r="AJ23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -1700,6 +1733,7 @@
       <c r="AG24" s="3" t="n"/>
       <c r="AH24" s="3" t="n"/>
       <c r="AI24" s="3" t="n"/>
+      <c r="AJ24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -1737,6 +1771,7 @@
       <c r="AG25" s="3" t="n"/>
       <c r="AH25" s="3" t="n"/>
       <c r="AI25" s="3" t="n"/>
+      <c r="AJ25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -1774,6 +1809,7 @@
       <c r="AG26" s="3" t="n"/>
       <c r="AH26" s="3" t="n"/>
       <c r="AI26" s="3" t="n"/>
+      <c r="AJ26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -1811,6 +1847,7 @@
       <c r="AG27" s="3" t="n"/>
       <c r="AH27" s="3" t="n"/>
       <c r="AI27" s="3" t="n"/>
+      <c r="AJ27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -1848,6 +1885,7 @@
       <c r="AG28" s="3" t="n"/>
       <c r="AH28" s="3" t="n"/>
       <c r="AI28" s="3" t="n"/>
+      <c r="AJ28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -1885,6 +1923,7 @@
       <c r="AG29" s="3" t="n"/>
       <c r="AH29" s="3" t="n"/>
       <c r="AI29" s="3" t="n"/>
+      <c r="AJ29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -1922,6 +1961,7 @@
       <c r="AG30" s="3" t="n"/>
       <c r="AH30" s="3" t="n"/>
       <c r="AI30" s="3" t="n"/>
+      <c r="AJ30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -1959,6 +1999,7 @@
       <c r="AG31" s="3" t="n"/>
       <c r="AH31" s="3" t="n"/>
       <c r="AI31" s="3" t="n"/>
+      <c r="AJ31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -1996,6 +2037,7 @@
       <c r="AG32" s="3" t="n"/>
       <c r="AH32" s="3" t="n"/>
       <c r="AI32" s="3" t="n"/>
+      <c r="AJ32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -2033,6 +2075,7 @@
       <c r="AG33" s="3" t="n"/>
       <c r="AH33" s="3" t="n"/>
       <c r="AI33" s="3" t="n"/>
+      <c r="AJ33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -2070,6 +2113,7 @@
       <c r="AG34" s="3" t="n"/>
       <c r="AH34" s="3" t="n"/>
       <c r="AI34" s="3" t="n"/>
+      <c r="AJ34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -2107,6 +2151,7 @@
       <c r="AG35" s="3" t="n"/>
       <c r="AH35" s="3" t="n"/>
       <c r="AI35" s="3" t="n"/>
+      <c r="AJ35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -2144,6 +2189,7 @@
       <c r="AG36" s="3" t="n"/>
       <c r="AH36" s="3" t="n"/>
       <c r="AI36" s="3" t="n"/>
+      <c r="AJ36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -2181,6 +2227,7 @@
       <c r="AG37" s="3" t="n"/>
       <c r="AH37" s="3" t="n"/>
       <c r="AI37" s="3" t="n"/>
+      <c r="AJ37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -2218,6 +2265,7 @@
       <c r="AG38" s="3" t="n"/>
       <c r="AH38" s="3" t="n"/>
       <c r="AI38" s="3" t="n"/>
+      <c r="AJ38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -2255,6 +2303,7 @@
       <c r="AG39" s="3" t="n"/>
       <c r="AH39" s="3" t="n"/>
       <c r="AI39" s="3" t="n"/>
+      <c r="AJ39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -2292,6 +2341,7 @@
       <c r="AG40" s="3" t="n"/>
       <c r="AH40" s="3" t="n"/>
       <c r="AI40" s="3" t="n"/>
+      <c r="AJ40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -2329,6 +2379,7 @@
       <c r="AG41" s="3" t="n"/>
       <c r="AH41" s="3" t="n"/>
       <c r="AI41" s="3" t="n"/>
+      <c r="AJ41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -2366,6 +2417,7 @@
       <c r="AG42" s="3" t="n"/>
       <c r="AH42" s="3" t="n"/>
       <c r="AI42" s="3" t="n"/>
+      <c r="AJ42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -2403,6 +2455,7 @@
       <c r="AG43" s="3" t="n"/>
       <c r="AH43" s="3" t="n"/>
       <c r="AI43" s="3" t="n"/>
+      <c r="AJ43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -2440,6 +2493,7 @@
       <c r="AG44" s="3" t="n"/>
       <c r="AH44" s="3" t="n"/>
       <c r="AI44" s="3" t="n"/>
+      <c r="AJ44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -2477,6 +2531,7 @@
       <c r="AG45" s="3" t="n"/>
       <c r="AH45" s="3" t="n"/>
       <c r="AI45" s="3" t="n"/>
+      <c r="AJ45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -2514,6 +2569,7 @@
       <c r="AG46" s="3" t="n"/>
       <c r="AH46" s="3" t="n"/>
       <c r="AI46" s="3" t="n"/>
+      <c r="AJ46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -2551,6 +2607,7 @@
       <c r="AG47" s="3" t="n"/>
       <c r="AH47" s="3" t="n"/>
       <c r="AI47" s="3" t="n"/>
+      <c r="AJ47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -2588,6 +2645,7 @@
       <c r="AG48" s="3" t="n"/>
       <c r="AH48" s="3" t="n"/>
       <c r="AI48" s="3" t="n"/>
+      <c r="AJ48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -2625,6 +2683,7 @@
       <c r="AG49" s="3" t="n"/>
       <c r="AH49" s="3" t="n"/>
       <c r="AI49" s="3" t="n"/>
+      <c r="AJ49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -2662,6 +2721,7 @@
       <c r="AG50" s="3" t="n"/>
       <c r="AH50" s="3" t="n"/>
       <c r="AI50" s="3" t="n"/>
+      <c r="AJ50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -2699,6 +2759,7 @@
       <c r="AG51" s="3" t="n"/>
       <c r="AH51" s="3" t="n"/>
       <c r="AI51" s="3" t="n"/>
+      <c r="AJ51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -2736,6 +2797,7 @@
       <c r="AG52" s="3" t="n"/>
       <c r="AH52" s="3" t="n"/>
       <c r="AI52" s="3" t="n"/>
+      <c r="AJ52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -2773,6 +2835,7 @@
       <c r="AG53" s="3" t="n"/>
       <c r="AH53" s="3" t="n"/>
       <c r="AI53" s="3" t="n"/>
+      <c r="AJ53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -2810,6 +2873,7 @@
       <c r="AG54" s="3" t="n"/>
       <c r="AH54" s="3" t="n"/>
       <c r="AI54" s="3" t="n"/>
+      <c r="AJ54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -2847,6 +2911,7 @@
       <c r="AG55" s="3" t="n"/>
       <c r="AH55" s="3" t="n"/>
       <c r="AI55" s="3" t="n"/>
+      <c r="AJ55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -2884,6 +2949,7 @@
       <c r="AG56" s="3" t="n"/>
       <c r="AH56" s="3" t="n"/>
       <c r="AI56" s="3" t="n"/>
+      <c r="AJ56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -2921,6 +2987,7 @@
       <c r="AG57" s="3" t="n"/>
       <c r="AH57" s="3" t="n"/>
       <c r="AI57" s="3" t="n"/>
+      <c r="AJ57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -2958,6 +3025,7 @@
       <c r="AG58" s="3" t="n"/>
       <c r="AH58" s="3" t="n"/>
       <c r="AI58" s="3" t="n"/>
+      <c r="AJ58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -2995,6 +3063,7 @@
       <c r="AG59" s="3" t="n"/>
       <c r="AH59" s="3" t="n"/>
       <c r="AI59" s="3" t="n"/>
+      <c r="AJ59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -3032,6 +3101,7 @@
       <c r="AG60" s="3" t="n"/>
       <c r="AH60" s="3" t="n"/>
       <c r="AI60" s="3" t="n"/>
+      <c r="AJ60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -3069,6 +3139,7 @@
       <c r="AG61" s="3" t="n"/>
       <c r="AH61" s="3" t="n"/>
       <c r="AI61" s="3" t="n"/>
+      <c r="AJ61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -3106,6 +3177,7 @@
       <c r="AG62" s="3" t="n"/>
       <c r="AH62" s="3" t="n"/>
       <c r="AI62" s="3" t="n"/>
+      <c r="AJ62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
@@ -3143,6 +3215,7 @@
       <c r="AG63" s="3" t="n"/>
       <c r="AH63" s="3" t="n"/>
       <c r="AI63" s="3" t="n"/>
+      <c r="AJ63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -3180,6 +3253,7 @@
       <c r="AG64" s="3" t="n"/>
       <c r="AH64" s="3" t="n"/>
       <c r="AI64" s="3" t="n"/>
+      <c r="AJ64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -3217,6 +3291,7 @@
       <c r="AG65" s="3" t="n"/>
       <c r="AH65" s="3" t="n"/>
       <c r="AI65" s="3" t="n"/>
+      <c r="AJ65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -3254,6 +3329,7 @@
       <c r="AG66" s="3" t="n"/>
       <c r="AH66" s="3" t="n"/>
       <c r="AI66" s="3" t="n"/>
+      <c r="AJ66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -3291,6 +3367,7 @@
       <c r="AG67" s="3" t="n"/>
       <c r="AH67" s="3" t="n"/>
       <c r="AI67" s="3" t="n"/>
+      <c r="AJ67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -3328,6 +3405,7 @@
       <c r="AG68" s="3" t="n"/>
       <c r="AH68" s="3" t="n"/>
       <c r="AI68" s="3" t="n"/>
+      <c r="AJ68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
@@ -3365,6 +3443,7 @@
       <c r="AG69" s="3" t="n"/>
       <c r="AH69" s="3" t="n"/>
       <c r="AI69" s="3" t="n"/>
+      <c r="AJ69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -3402,6 +3481,7 @@
       <c r="AG70" s="3" t="n"/>
       <c r="AH70" s="3" t="n"/>
       <c r="AI70" s="3" t="n"/>
+      <c r="AJ70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
@@ -3439,6 +3519,7 @@
       <c r="AG71" s="3" t="n"/>
       <c r="AH71" s="3" t="n"/>
       <c r="AI71" s="3" t="n"/>
+      <c r="AJ71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -3476,6 +3557,7 @@
       <c r="AG72" s="3" t="n"/>
       <c r="AH72" s="3" t="n"/>
       <c r="AI72" s="3" t="n"/>
+      <c r="AJ72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
@@ -3513,6 +3595,7 @@
       <c r="AG73" s="3" t="n"/>
       <c r="AH73" s="3" t="n"/>
       <c r="AI73" s="3" t="n"/>
+      <c r="AJ73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -3550,6 +3633,7 @@
       <c r="AG74" s="3" t="n"/>
       <c r="AH74" s="3" t="n"/>
       <c r="AI74" s="3" t="n"/>
+      <c r="AJ74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
@@ -3587,6 +3671,7 @@
       <c r="AG75" s="3" t="n"/>
       <c r="AH75" s="3" t="n"/>
       <c r="AI75" s="3" t="n"/>
+      <c r="AJ75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -3624,6 +3709,7 @@
       <c r="AG76" s="3" t="n"/>
       <c r="AH76" s="3" t="n"/>
       <c r="AI76" s="3" t="n"/>
+      <c r="AJ76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -3661,6 +3747,7 @@
       <c r="AG77" s="3" t="n"/>
       <c r="AH77" s="3" t="n"/>
       <c r="AI77" s="3" t="n"/>
+      <c r="AJ77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -3698,6 +3785,7 @@
       <c r="AG78" s="3" t="n"/>
       <c r="AH78" s="3" t="n"/>
       <c r="AI78" s="3" t="n"/>
+      <c r="AJ78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
@@ -3735,6 +3823,7 @@
       <c r="AG79" s="3" t="n"/>
       <c r="AH79" s="3" t="n"/>
       <c r="AI79" s="3" t="n"/>
+      <c r="AJ79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -3772,6 +3861,7 @@
       <c r="AG80" s="3" t="n"/>
       <c r="AH80" s="3" t="n"/>
       <c r="AI80" s="3" t="n"/>
+      <c r="AJ80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
@@ -3809,6 +3899,7 @@
       <c r="AG81" s="3" t="n"/>
       <c r="AH81" s="3" t="n"/>
       <c r="AI81" s="3" t="n"/>
+      <c r="AJ81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -3846,6 +3937,7 @@
       <c r="AG82" s="3" t="n"/>
       <c r="AH82" s="3" t="n"/>
       <c r="AI82" s="3" t="n"/>
+      <c r="AJ82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n"/>
@@ -3883,6 +3975,7 @@
       <c r="AG83" s="3" t="n"/>
       <c r="AH83" s="3" t="n"/>
       <c r="AI83" s="3" t="n"/>
+      <c r="AJ83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -3920,6 +4013,7 @@
       <c r="AG84" s="3" t="n"/>
       <c r="AH84" s="3" t="n"/>
       <c r="AI84" s="3" t="n"/>
+      <c r="AJ84" s="3" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n"/>
@@ -3957,6 +4051,7 @@
       <c r="AG85" s="3" t="n"/>
       <c r="AH85" s="3" t="n"/>
       <c r="AI85" s="3" t="n"/>
+      <c r="AJ85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -3994,6 +4089,7 @@
       <c r="AG86" s="3" t="n"/>
       <c r="AH86" s="3" t="n"/>
       <c r="AI86" s="3" t="n"/>
+      <c r="AJ86" s="3" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n"/>
@@ -4031,6 +4127,7 @@
       <c r="AG87" s="3" t="n"/>
       <c r="AH87" s="3" t="n"/>
       <c r="AI87" s="3" t="n"/>
+      <c r="AJ87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -4068,6 +4165,7 @@
       <c r="AG88" s="3" t="n"/>
       <c r="AH88" s="3" t="n"/>
       <c r="AI88" s="3" t="n"/>
+      <c r="AJ88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n"/>
@@ -4105,6 +4203,7 @@
       <c r="AG89" s="3" t="n"/>
       <c r="AH89" s="3" t="n"/>
       <c r="AI89" s="3" t="n"/>
+      <c r="AJ89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -4142,6 +4241,7 @@
       <c r="AG90" s="3" t="n"/>
       <c r="AH90" s="3" t="n"/>
       <c r="AI90" s="3" t="n"/>
+      <c r="AJ90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n"/>
@@ -4179,6 +4279,7 @@
       <c r="AG91" s="3" t="n"/>
       <c r="AH91" s="3" t="n"/>
       <c r="AI91" s="3" t="n"/>
+      <c r="AJ91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -4216,6 +4317,7 @@
       <c r="AG92" s="3" t="n"/>
       <c r="AH92" s="3" t="n"/>
       <c r="AI92" s="3" t="n"/>
+      <c r="AJ92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n"/>
@@ -4253,6 +4355,7 @@
       <c r="AG93" s="3" t="n"/>
       <c r="AH93" s="3" t="n"/>
       <c r="AI93" s="3" t="n"/>
+      <c r="AJ93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -4290,6 +4393,7 @@
       <c r="AG94" s="3" t="n"/>
       <c r="AH94" s="3" t="n"/>
       <c r="AI94" s="3" t="n"/>
+      <c r="AJ94" s="3" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n"/>
@@ -4327,6 +4431,7 @@
       <c r="AG95" s="3" t="n"/>
       <c r="AH95" s="3" t="n"/>
       <c r="AI95" s="3" t="n"/>
+      <c r="AJ95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -4364,6 +4469,7 @@
       <c r="AG96" s="3" t="n"/>
       <c r="AH96" s="3" t="n"/>
       <c r="AI96" s="3" t="n"/>
+      <c r="AJ96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n"/>
@@ -4401,6 +4507,7 @@
       <c r="AG97" s="3" t="n"/>
       <c r="AH97" s="3" t="n"/>
       <c r="AI97" s="3" t="n"/>
+      <c r="AJ97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -4438,6 +4545,7 @@
       <c r="AG98" s="3" t="n"/>
       <c r="AH98" s="3" t="n"/>
       <c r="AI98" s="3" t="n"/>
+      <c r="AJ98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n"/>
@@ -4475,6 +4583,7 @@
       <c r="AG99" s="3" t="n"/>
       <c r="AH99" s="3" t="n"/>
       <c r="AI99" s="3" t="n"/>
+      <c r="AJ99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -4512,6 +4621,7 @@
       <c r="AG100" s="3" t="n"/>
       <c r="AH100" s="3" t="n"/>
       <c r="AI100" s="3" t="n"/>
+      <c r="AJ100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n"/>
@@ -4549,6 +4659,7 @@
       <c r="AG101" s="3" t="n"/>
       <c r="AH101" s="3" t="n"/>
       <c r="AI101" s="3" t="n"/>
+      <c r="AJ101" s="3" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n"/>
@@ -4586,6 +4697,7 @@
       <c r="AG102" s="3" t="n"/>
       <c r="AH102" s="3" t="n"/>
       <c r="AI102" s="3" t="n"/>
+      <c r="AJ102" s="3" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n"/>
@@ -4623,6 +4735,7 @@
       <c r="AG103" s="3" t="n"/>
       <c r="AH103" s="3" t="n"/>
       <c r="AI103" s="3" t="n"/>
+      <c r="AJ103" s="3" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n"/>
@@ -4660,6 +4773,7 @@
       <c r="AG104" s="3" t="n"/>
       <c r="AH104" s="3" t="n"/>
       <c r="AI104" s="3" t="n"/>
+      <c r="AJ104" s="3" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n"/>
@@ -4697,6 +4811,7 @@
       <c r="AG105" s="3" t="n"/>
       <c r="AH105" s="3" t="n"/>
       <c r="AI105" s="3" t="n"/>
+      <c r="AJ105" s="3" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n"/>
@@ -4734,6 +4849,7 @@
       <c r="AG106" s="3" t="n"/>
       <c r="AH106" s="3" t="n"/>
       <c r="AI106" s="3" t="n"/>
+      <c r="AJ106" s="3" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n"/>
@@ -4771,6 +4887,7 @@
       <c r="AG107" s="3" t="n"/>
       <c r="AH107" s="3" t="n"/>
       <c r="AI107" s="3" t="n"/>
+      <c r="AJ107" s="3" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n"/>
@@ -4808,6 +4925,7 @@
       <c r="AG108" s="3" t="n"/>
       <c r="AH108" s="3" t="n"/>
       <c r="AI108" s="3" t="n"/>
+      <c r="AJ108" s="3" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n"/>
@@ -4845,6 +4963,7 @@
       <c r="AG109" s="3" t="n"/>
       <c r="AH109" s="3" t="n"/>
       <c r="AI109" s="3" t="n"/>
+      <c r="AJ109" s="3" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n"/>
@@ -4882,6 +5001,7 @@
       <c r="AG110" s="3" t="n"/>
       <c r="AH110" s="3" t="n"/>
       <c r="AI110" s="3" t="n"/>
+      <c r="AJ110" s="3" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n"/>
@@ -4919,6 +5039,7 @@
       <c r="AG111" s="3" t="n"/>
       <c r="AH111" s="3" t="n"/>
       <c r="AI111" s="3" t="n"/>
+      <c r="AJ111" s="3" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="3" t="n"/>
@@ -4956,6 +5077,7 @@
       <c r="AG112" s="3" t="n"/>
       <c r="AH112" s="3" t="n"/>
       <c r="AI112" s="3" t="n"/>
+      <c r="AJ112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n"/>
@@ -4993,6 +5115,7 @@
       <c r="AG113" s="3" t="n"/>
       <c r="AH113" s="3" t="n"/>
       <c r="AI113" s="3" t="n"/>
+      <c r="AJ113" s="3" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n"/>
@@ -5030,6 +5153,7 @@
       <c r="AG114" s="3" t="n"/>
       <c r="AH114" s="3" t="n"/>
       <c r="AI114" s="3" t="n"/>
+      <c r="AJ114" s="3" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n"/>
@@ -5067,6 +5191,7 @@
       <c r="AG115" s="3" t="n"/>
       <c r="AH115" s="3" t="n"/>
       <c r="AI115" s="3" t="n"/>
+      <c r="AJ115" s="3" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n"/>
@@ -5104,6 +5229,7 @@
       <c r="AG116" s="3" t="n"/>
       <c r="AH116" s="3" t="n"/>
       <c r="AI116" s="3" t="n"/>
+      <c r="AJ116" s="3" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="3" t="n"/>
@@ -5141,6 +5267,7 @@
       <c r="AG117" s="3" t="n"/>
       <c r="AH117" s="3" t="n"/>
       <c r="AI117" s="3" t="n"/>
+      <c r="AJ117" s="3" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n"/>
@@ -5178,6 +5305,7 @@
       <c r="AG118" s="3" t="n"/>
       <c r="AH118" s="3" t="n"/>
       <c r="AI118" s="3" t="n"/>
+      <c r="AJ118" s="3" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="n"/>
@@ -5215,6 +5343,7 @@
       <c r="AG119" s="3" t="n"/>
       <c r="AH119" s="3" t="n"/>
       <c r="AI119" s="3" t="n"/>
+      <c r="AJ119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="n"/>
@@ -5252,6 +5381,7 @@
       <c r="AG120" s="3" t="n"/>
       <c r="AH120" s="3" t="n"/>
       <c r="AI120" s="3" t="n"/>
+      <c r="AJ120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="n"/>
@@ -5289,6 +5419,7 @@
       <c r="AG121" s="3" t="n"/>
       <c r="AH121" s="3" t="n"/>
       <c r="AI121" s="3" t="n"/>
+      <c r="AJ121" s="3" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n"/>
@@ -5326,6 +5457,7 @@
       <c r="AG122" s="3" t="n"/>
       <c r="AH122" s="3" t="n"/>
       <c r="AI122" s="3" t="n"/>
+      <c r="AJ122" s="3" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="n"/>
@@ -5363,6 +5495,7 @@
       <c r="AG123" s="3" t="n"/>
       <c r="AH123" s="3" t="n"/>
       <c r="AI123" s="3" t="n"/>
+      <c r="AJ123" s="3" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n"/>
@@ -5400,6 +5533,7 @@
       <c r="AG124" s="3" t="n"/>
       <c r="AH124" s="3" t="n"/>
       <c r="AI124" s="3" t="n"/>
+      <c r="AJ124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n"/>
@@ -5437,6 +5571,7 @@
       <c r="AG125" s="3" t="n"/>
       <c r="AH125" s="3" t="n"/>
       <c r="AI125" s="3" t="n"/>
+      <c r="AJ125" s="3" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n"/>
@@ -5474,6 +5609,7 @@
       <c r="AG126" s="3" t="n"/>
       <c r="AH126" s="3" t="n"/>
       <c r="AI126" s="3" t="n"/>
+      <c r="AJ126" s="3" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="3" t="n"/>
@@ -5511,6 +5647,7 @@
       <c r="AG127" s="3" t="n"/>
       <c r="AH127" s="3" t="n"/>
       <c r="AI127" s="3" t="n"/>
+      <c r="AJ127" s="3" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="n"/>
@@ -5548,6 +5685,7 @@
       <c r="AG128" s="3" t="n"/>
       <c r="AH128" s="3" t="n"/>
       <c r="AI128" s="3" t="n"/>
+      <c r="AJ128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="3" t="n"/>
@@ -5585,6 +5723,7 @@
       <c r="AG129" s="3" t="n"/>
       <c r="AH129" s="3" t="n"/>
       <c r="AI129" s="3" t="n"/>
+      <c r="AJ129" s="3" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n"/>
@@ -5622,6 +5761,7 @@
       <c r="AG130" s="3" t="n"/>
       <c r="AH130" s="3" t="n"/>
       <c r="AI130" s="3" t="n"/>
+      <c r="AJ130" s="3" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="n"/>
@@ -5659,6 +5799,7 @@
       <c r="AG131" s="3" t="n"/>
       <c r="AH131" s="3" t="n"/>
       <c r="AI131" s="3" t="n"/>
+      <c r="AJ131" s="3" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n"/>
@@ -5696,6 +5837,7 @@
       <c r="AG132" s="3" t="n"/>
       <c r="AH132" s="3" t="n"/>
       <c r="AI132" s="3" t="n"/>
+      <c r="AJ132" s="3" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="3" t="n"/>
@@ -5733,6 +5875,7 @@
       <c r="AG133" s="3" t="n"/>
       <c r="AH133" s="3" t="n"/>
       <c r="AI133" s="3" t="n"/>
+      <c r="AJ133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="3" t="n"/>
@@ -5770,6 +5913,7 @@
       <c r="AG134" s="3" t="n"/>
       <c r="AH134" s="3" t="n"/>
       <c r="AI134" s="3" t="n"/>
+      <c r="AJ134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="3" t="n"/>
@@ -5807,6 +5951,7 @@
       <c r="AG135" s="3" t="n"/>
       <c r="AH135" s="3" t="n"/>
       <c r="AI135" s="3" t="n"/>
+      <c r="AJ135" s="3" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="n"/>
@@ -5844,6 +5989,7 @@
       <c r="AG136" s="3" t="n"/>
       <c r="AH136" s="3" t="n"/>
       <c r="AI136" s="3" t="n"/>
+      <c r="AJ136" s="3" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="3" t="n"/>
@@ -5881,6 +6027,7 @@
       <c r="AG137" s="3" t="n"/>
       <c r="AH137" s="3" t="n"/>
       <c r="AI137" s="3" t="n"/>
+      <c r="AJ137" s="3" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="3" t="n"/>
@@ -5918,6 +6065,7 @@
       <c r="AG138" s="3" t="n"/>
       <c r="AH138" s="3" t="n"/>
       <c r="AI138" s="3" t="n"/>
+      <c r="AJ138" s="3" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="3" t="n"/>
@@ -5955,6 +6103,7 @@
       <c r="AG139" s="3" t="n"/>
       <c r="AH139" s="3" t="n"/>
       <c r="AI139" s="3" t="n"/>
+      <c r="AJ139" s="3" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n"/>
@@ -5992,6 +6141,7 @@
       <c r="AG140" s="3" t="n"/>
       <c r="AH140" s="3" t="n"/>
       <c r="AI140" s="3" t="n"/>
+      <c r="AJ140" s="3" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="3" t="n"/>
@@ -6029,6 +6179,7 @@
       <c r="AG141" s="3" t="n"/>
       <c r="AH141" s="3" t="n"/>
       <c r="AI141" s="3" t="n"/>
+      <c r="AJ141" s="3" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="3" t="n"/>
@@ -6066,6 +6217,7 @@
       <c r="AG142" s="3" t="n"/>
       <c r="AH142" s="3" t="n"/>
       <c r="AI142" s="3" t="n"/>
+      <c r="AJ142" s="3" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="3" t="n"/>
@@ -6103,6 +6255,7 @@
       <c r="AG143" s="3" t="n"/>
       <c r="AH143" s="3" t="n"/>
       <c r="AI143" s="3" t="n"/>
+      <c r="AJ143" s="3" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="3" t="n"/>
@@ -6140,6 +6293,7 @@
       <c r="AG144" s="3" t="n"/>
       <c r="AH144" s="3" t="n"/>
       <c r="AI144" s="3" t="n"/>
+      <c r="AJ144" s="3" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="3" t="n"/>
@@ -6177,6 +6331,7 @@
       <c r="AG145" s="3" t="n"/>
       <c r="AH145" s="3" t="n"/>
       <c r="AI145" s="3" t="n"/>
+      <c r="AJ145" s="3" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="3" t="n"/>
@@ -6214,6 +6369,7 @@
       <c r="AG146" s="3" t="n"/>
       <c r="AH146" s="3" t="n"/>
       <c r="AI146" s="3" t="n"/>
+      <c r="AJ146" s="3" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="n"/>
@@ -6251,6 +6407,7 @@
       <c r="AG147" s="3" t="n"/>
       <c r="AH147" s="3" t="n"/>
       <c r="AI147" s="3" t="n"/>
+      <c r="AJ147" s="3" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="3" t="n"/>
@@ -6288,6 +6445,7 @@
       <c r="AG148" s="3" t="n"/>
       <c r="AH148" s="3" t="n"/>
       <c r="AI148" s="3" t="n"/>
+      <c r="AJ148" s="3" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="3" t="n"/>
@@ -6325,6 +6483,7 @@
       <c r="AG149" s="3" t="n"/>
       <c r="AH149" s="3" t="n"/>
       <c r="AI149" s="3" t="n"/>
+      <c r="AJ149" s="3" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="3" t="n"/>
@@ -6362,6 +6521,7 @@
       <c r="AG150" s="3" t="n"/>
       <c r="AH150" s="3" t="n"/>
       <c r="AI150" s="3" t="n"/>
+      <c r="AJ150" s="3" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="3" t="n"/>
@@ -6399,6 +6559,7 @@
       <c r="AG151" s="3" t="n"/>
       <c r="AH151" s="3" t="n"/>
       <c r="AI151" s="3" t="n"/>
+      <c r="AJ151" s="3" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="3" t="n"/>
@@ -6436,6 +6597,7 @@
       <c r="AG152" s="3" t="n"/>
       <c r="AH152" s="3" t="n"/>
       <c r="AI152" s="3" t="n"/>
+      <c r="AJ152" s="3" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="n"/>
@@ -6473,6 +6635,7 @@
       <c r="AG153" s="3" t="n"/>
       <c r="AH153" s="3" t="n"/>
       <c r="AI153" s="3" t="n"/>
+      <c r="AJ153" s="3" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="n"/>
@@ -6510,6 +6673,7 @@
       <c r="AG154" s="3" t="n"/>
       <c r="AH154" s="3" t="n"/>
       <c r="AI154" s="3" t="n"/>
+      <c r="AJ154" s="3" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="3" t="n"/>
@@ -6547,6 +6711,7 @@
       <c r="AG155" s="3" t="n"/>
       <c r="AH155" s="3" t="n"/>
       <c r="AI155" s="3" t="n"/>
+      <c r="AJ155" s="3" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="n"/>
@@ -6584,6 +6749,7 @@
       <c r="AG156" s="3" t="n"/>
       <c r="AH156" s="3" t="n"/>
       <c r="AI156" s="3" t="n"/>
+      <c r="AJ156" s="3" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="3" t="n"/>
@@ -6621,6 +6787,7 @@
       <c r="AG157" s="3" t="n"/>
       <c r="AH157" s="3" t="n"/>
       <c r="AI157" s="3" t="n"/>
+      <c r="AJ157" s="3" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="3" t="n"/>
@@ -6658,6 +6825,7 @@
       <c r="AG158" s="3" t="n"/>
       <c r="AH158" s="3" t="n"/>
       <c r="AI158" s="3" t="n"/>
+      <c r="AJ158" s="3" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="3" t="n"/>
@@ -6695,6 +6863,7 @@
       <c r="AG159" s="3" t="n"/>
       <c r="AH159" s="3" t="n"/>
       <c r="AI159" s="3" t="n"/>
+      <c r="AJ159" s="3" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="3" t="n"/>
@@ -6732,6 +6901,7 @@
       <c r="AG160" s="3" t="n"/>
       <c r="AH160" s="3" t="n"/>
       <c r="AI160" s="3" t="n"/>
+      <c r="AJ160" s="3" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="3" t="n"/>
@@ -6769,6 +6939,7 @@
       <c r="AG161" s="3" t="n"/>
       <c r="AH161" s="3" t="n"/>
       <c r="AI161" s="3" t="n"/>
+      <c r="AJ161" s="3" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="3" t="n"/>
@@ -6806,6 +6977,7 @@
       <c r="AG162" s="3" t="n"/>
       <c r="AH162" s="3" t="n"/>
       <c r="AI162" s="3" t="n"/>
+      <c r="AJ162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="3" t="n"/>
@@ -6843,6 +7015,7 @@
       <c r="AG163" s="3" t="n"/>
       <c r="AH163" s="3" t="n"/>
       <c r="AI163" s="3" t="n"/>
+      <c r="AJ163" s="3" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="3" t="n"/>
@@ -6880,6 +7053,7 @@
       <c r="AG164" s="3" t="n"/>
       <c r="AH164" s="3" t="n"/>
       <c r="AI164" s="3" t="n"/>
+      <c r="AJ164" s="3" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="3" t="n"/>
@@ -6917,6 +7091,7 @@
       <c r="AG165" s="3" t="n"/>
       <c r="AH165" s="3" t="n"/>
       <c r="AI165" s="3" t="n"/>
+      <c r="AJ165" s="3" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="3" t="n"/>
@@ -6954,6 +7129,7 @@
       <c r="AG166" s="3" t="n"/>
       <c r="AH166" s="3" t="n"/>
       <c r="AI166" s="3" t="n"/>
+      <c r="AJ166" s="3" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="3" t="n"/>
@@ -6991,6 +7167,7 @@
       <c r="AG167" s="3" t="n"/>
       <c r="AH167" s="3" t="n"/>
       <c r="AI167" s="3" t="n"/>
+      <c r="AJ167" s="3" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="3" t="n"/>
@@ -7028,6 +7205,7 @@
       <c r="AG168" s="3" t="n"/>
       <c r="AH168" s="3" t="n"/>
       <c r="AI168" s="3" t="n"/>
+      <c r="AJ168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="3" t="n"/>
@@ -7065,6 +7243,7 @@
       <c r="AG169" s="3" t="n"/>
       <c r="AH169" s="3" t="n"/>
       <c r="AI169" s="3" t="n"/>
+      <c r="AJ169" s="3" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="n"/>
@@ -7102,6 +7281,7 @@
       <c r="AG170" s="3" t="n"/>
       <c r="AH170" s="3" t="n"/>
       <c r="AI170" s="3" t="n"/>
+      <c r="AJ170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="3" t="n"/>
@@ -7139,6 +7319,7 @@
       <c r="AG171" s="3" t="n"/>
       <c r="AH171" s="3" t="n"/>
       <c r="AI171" s="3" t="n"/>
+      <c r="AJ171" s="3" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="3" t="n"/>
@@ -7176,6 +7357,7 @@
       <c r="AG172" s="3" t="n"/>
       <c r="AH172" s="3" t="n"/>
       <c r="AI172" s="3" t="n"/>
+      <c r="AJ172" s="3" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="3" t="n"/>
@@ -7213,6 +7395,7 @@
       <c r="AG173" s="3" t="n"/>
       <c r="AH173" s="3" t="n"/>
       <c r="AI173" s="3" t="n"/>
+      <c r="AJ173" s="3" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="3" t="n"/>
@@ -7250,6 +7433,7 @@
       <c r="AG174" s="3" t="n"/>
       <c r="AH174" s="3" t="n"/>
       <c r="AI174" s="3" t="n"/>
+      <c r="AJ174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="3" t="n"/>
@@ -7287,6 +7471,7 @@
       <c r="AG175" s="3" t="n"/>
       <c r="AH175" s="3" t="n"/>
       <c r="AI175" s="3" t="n"/>
+      <c r="AJ175" s="3" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="3" t="n"/>
@@ -7324,6 +7509,7 @@
       <c r="AG176" s="3" t="n"/>
       <c r="AH176" s="3" t="n"/>
       <c r="AI176" s="3" t="n"/>
+      <c r="AJ176" s="3" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="3" t="n"/>
@@ -7361,6 +7547,7 @@
       <c r="AG177" s="3" t="n"/>
       <c r="AH177" s="3" t="n"/>
       <c r="AI177" s="3" t="n"/>
+      <c r="AJ177" s="3" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="n"/>
@@ -7398,6 +7585,7 @@
       <c r="AG178" s="3" t="n"/>
       <c r="AH178" s="3" t="n"/>
       <c r="AI178" s="3" t="n"/>
+      <c r="AJ178" s="3" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="3" t="n"/>
@@ -7435,6 +7623,7 @@
       <c r="AG179" s="3" t="n"/>
       <c r="AH179" s="3" t="n"/>
       <c r="AI179" s="3" t="n"/>
+      <c r="AJ179" s="3" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="3" t="n"/>
@@ -7472,6 +7661,7 @@
       <c r="AG180" s="3" t="n"/>
       <c r="AH180" s="3" t="n"/>
       <c r="AI180" s="3" t="n"/>
+      <c r="AJ180" s="3" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="3" t="n"/>
@@ -7509,6 +7699,7 @@
       <c r="AG181" s="3" t="n"/>
       <c r="AH181" s="3" t="n"/>
       <c r="AI181" s="3" t="n"/>
+      <c r="AJ181" s="3" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="3" t="n"/>
@@ -7546,6 +7737,7 @@
       <c r="AG182" s="3" t="n"/>
       <c r="AH182" s="3" t="n"/>
       <c r="AI182" s="3" t="n"/>
+      <c r="AJ182" s="3" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="n"/>
@@ -7583,6 +7775,7 @@
       <c r="AG183" s="3" t="n"/>
       <c r="AH183" s="3" t="n"/>
       <c r="AI183" s="3" t="n"/>
+      <c r="AJ183" s="3" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="n"/>
@@ -7620,6 +7813,7 @@
       <c r="AG184" s="3" t="n"/>
       <c r="AH184" s="3" t="n"/>
       <c r="AI184" s="3" t="n"/>
+      <c r="AJ184" s="3" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="n"/>
@@ -7657,6 +7851,7 @@
       <c r="AG185" s="3" t="n"/>
       <c r="AH185" s="3" t="n"/>
       <c r="AI185" s="3" t="n"/>
+      <c r="AJ185" s="3" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="3" t="n"/>
@@ -7694,6 +7889,7 @@
       <c r="AG186" s="3" t="n"/>
       <c r="AH186" s="3" t="n"/>
       <c r="AI186" s="3" t="n"/>
+      <c r="AJ186" s="3" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="n"/>
@@ -7731,6 +7927,7 @@
       <c r="AG187" s="3" t="n"/>
       <c r="AH187" s="3" t="n"/>
       <c r="AI187" s="3" t="n"/>
+      <c r="AJ187" s="3" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="3" t="n"/>
@@ -7768,6 +7965,7 @@
       <c r="AG188" s="3" t="n"/>
       <c r="AH188" s="3" t="n"/>
       <c r="AI188" s="3" t="n"/>
+      <c r="AJ188" s="3" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="3" t="n"/>
@@ -7805,6 +8003,7 @@
       <c r="AG189" s="3" t="n"/>
       <c r="AH189" s="3" t="n"/>
       <c r="AI189" s="3" t="n"/>
+      <c r="AJ189" s="3" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="3" t="n"/>
@@ -7842,6 +8041,7 @@
       <c r="AG190" s="3" t="n"/>
       <c r="AH190" s="3" t="n"/>
       <c r="AI190" s="3" t="n"/>
+      <c r="AJ190" s="3" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="3" t="n"/>
@@ -7879,6 +8079,7 @@
       <c r="AG191" s="3" t="n"/>
       <c r="AH191" s="3" t="n"/>
       <c r="AI191" s="3" t="n"/>
+      <c r="AJ191" s="3" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n"/>
@@ -7916,6 +8117,7 @@
       <c r="AG192" s="3" t="n"/>
       <c r="AH192" s="3" t="n"/>
       <c r="AI192" s="3" t="n"/>
+      <c r="AJ192" s="3" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="3" t="n"/>
@@ -7953,6 +8155,7 @@
       <c r="AG193" s="3" t="n"/>
       <c r="AH193" s="3" t="n"/>
       <c r="AI193" s="3" t="n"/>
+      <c r="AJ193" s="3" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="3" t="n"/>
@@ -7990,6 +8193,7 @@
       <c r="AG194" s="3" t="n"/>
       <c r="AH194" s="3" t="n"/>
       <c r="AI194" s="3" t="n"/>
+      <c r="AJ194" s="3" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="3" t="n"/>
@@ -8027,6 +8231,7 @@
       <c r="AG195" s="3" t="n"/>
       <c r="AH195" s="3" t="n"/>
       <c r="AI195" s="3" t="n"/>
+      <c r="AJ195" s="3" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="3" t="n"/>
@@ -8064,6 +8269,7 @@
       <c r="AG196" s="3" t="n"/>
       <c r="AH196" s="3" t="n"/>
       <c r="AI196" s="3" t="n"/>
+      <c r="AJ196" s="3" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="3" t="n"/>
@@ -8101,6 +8307,7 @@
       <c r="AG197" s="3" t="n"/>
       <c r="AH197" s="3" t="n"/>
       <c r="AI197" s="3" t="n"/>
+      <c r="AJ197" s="3" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="3" t="n"/>
@@ -8138,6 +8345,7 @@
       <c r="AG198" s="3" t="n"/>
       <c r="AH198" s="3" t="n"/>
       <c r="AI198" s="3" t="n"/>
+      <c r="AJ198" s="3" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="3" t="n"/>
@@ -8175,6 +8383,7 @@
       <c r="AG199" s="3" t="n"/>
       <c r="AH199" s="3" t="n"/>
       <c r="AI199" s="3" t="n"/>
+      <c r="AJ199" s="3" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="3" t="n"/>
@@ -8212,6 +8421,7 @@
       <c r="AG200" s="3" t="n"/>
       <c r="AH200" s="3" t="n"/>
       <c r="AI200" s="3" t="n"/>
+      <c r="AJ200" s="3" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="3" t="n"/>
@@ -8249,6 +8459,7 @@
       <c r="AG201" s="3" t="n"/>
       <c r="AH201" s="3" t="n"/>
       <c r="AI201" s="3" t="n"/>
+      <c r="AJ201" s="3" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="3" t="n"/>
@@ -8286,6 +8497,7 @@
       <c r="AG202" s="3" t="n"/>
       <c r="AH202" s="3" t="n"/>
       <c r="AI202" s="3" t="n"/>
+      <c r="AJ202" s="3" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="3" t="n"/>
@@ -8323,6 +8535,7 @@
       <c r="AG203" s="3" t="n"/>
       <c r="AH203" s="3" t="n"/>
       <c r="AI203" s="3" t="n"/>
+      <c r="AJ203" s="3" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="3" t="n"/>
@@ -8360,6 +8573,7 @@
       <c r="AG204" s="3" t="n"/>
       <c r="AH204" s="3" t="n"/>
       <c r="AI204" s="3" t="n"/>
+      <c r="AJ204" s="3" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="3" t="n"/>
@@ -8397,6 +8611,7 @@
       <c r="AG205" s="3" t="n"/>
       <c r="AH205" s="3" t="n"/>
       <c r="AI205" s="3" t="n"/>
+      <c r="AJ205" s="3" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="3" t="n"/>
@@ -8434,6 +8649,7 @@
       <c r="AG206" s="3" t="n"/>
       <c r="AH206" s="3" t="n"/>
       <c r="AI206" s="3" t="n"/>
+      <c r="AJ206" s="3" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="3" t="n"/>
@@ -8471,6 +8687,7 @@
       <c r="AG207" s="3" t="n"/>
       <c r="AH207" s="3" t="n"/>
       <c r="AI207" s="3" t="n"/>
+      <c r="AJ207" s="3" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="3" t="n"/>
@@ -8508,6 +8725,7 @@
       <c r="AG208" s="3" t="n"/>
       <c r="AH208" s="3" t="n"/>
       <c r="AI208" s="3" t="n"/>
+      <c r="AJ208" s="3" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="3" t="n"/>
@@ -8545,6 +8763,7 @@
       <c r="AG209" s="3" t="n"/>
       <c r="AH209" s="3" t="n"/>
       <c r="AI209" s="3" t="n"/>
+      <c r="AJ209" s="3" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="3" t="n"/>
@@ -8582,6 +8801,7 @@
       <c r="AG210" s="3" t="n"/>
       <c r="AH210" s="3" t="n"/>
       <c r="AI210" s="3" t="n"/>
+      <c r="AJ210" s="3" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="3" t="n"/>
@@ -8619,6 +8839,7 @@
       <c r="AG211" s="3" t="n"/>
       <c r="AH211" s="3" t="n"/>
       <c r="AI211" s="3" t="n"/>
+      <c r="AJ211" s="3" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="3" t="n"/>
@@ -8656,6 +8877,7 @@
       <c r="AG212" s="3" t="n"/>
       <c r="AH212" s="3" t="n"/>
       <c r="AI212" s="3" t="n"/>
+      <c r="AJ212" s="3" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="3" t="n"/>
@@ -8693,6 +8915,7 @@
       <c r="AG213" s="3" t="n"/>
       <c r="AH213" s="3" t="n"/>
       <c r="AI213" s="3" t="n"/>
+      <c r="AJ213" s="3" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="3" t="n"/>
@@ -8730,6 +8953,7 @@
       <c r="AG214" s="3" t="n"/>
       <c r="AH214" s="3" t="n"/>
       <c r="AI214" s="3" t="n"/>
+      <c r="AJ214" s="3" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="3" t="n"/>
@@ -8767,6 +8991,7 @@
       <c r="AG215" s="3" t="n"/>
       <c r="AH215" s="3" t="n"/>
       <c r="AI215" s="3" t="n"/>
+      <c r="AJ215" s="3" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="3" t="n"/>
@@ -8804,6 +9029,7 @@
       <c r="AG216" s="3" t="n"/>
       <c r="AH216" s="3" t="n"/>
       <c r="AI216" s="3" t="n"/>
+      <c r="AJ216" s="3" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="3" t="n"/>
@@ -8841,6 +9067,7 @@
       <c r="AG217" s="3" t="n"/>
       <c r="AH217" s="3" t="n"/>
       <c r="AI217" s="3" t="n"/>
+      <c r="AJ217" s="3" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="3" t="n"/>
@@ -8878,6 +9105,7 @@
       <c r="AG218" s="3" t="n"/>
       <c r="AH218" s="3" t="n"/>
       <c r="AI218" s="3" t="n"/>
+      <c r="AJ218" s="3" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="3" t="n"/>
@@ -8915,6 +9143,7 @@
       <c r="AG219" s="3" t="n"/>
       <c r="AH219" s="3" t="n"/>
       <c r="AI219" s="3" t="n"/>
+      <c r="AJ219" s="3" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="3" t="n"/>
@@ -8952,6 +9181,7 @@
       <c r="AG220" s="3" t="n"/>
       <c r="AH220" s="3" t="n"/>
       <c r="AI220" s="3" t="n"/>
+      <c r="AJ220" s="3" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="3" t="n"/>
@@ -8989,6 +9219,7 @@
       <c r="AG221" s="3" t="n"/>
       <c r="AH221" s="3" t="n"/>
       <c r="AI221" s="3" t="n"/>
+      <c r="AJ221" s="3" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="3" t="n"/>
@@ -9026,6 +9257,7 @@
       <c r="AG222" s="3" t="n"/>
       <c r="AH222" s="3" t="n"/>
       <c r="AI222" s="3" t="n"/>
+      <c r="AJ222" s="3" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="3" t="n"/>
@@ -9063,6 +9295,7 @@
       <c r="AG223" s="3" t="n"/>
       <c r="AH223" s="3" t="n"/>
       <c r="AI223" s="3" t="n"/>
+      <c r="AJ223" s="3" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="3" t="n"/>
@@ -9100,6 +9333,7 @@
       <c r="AG224" s="3" t="n"/>
       <c r="AH224" s="3" t="n"/>
       <c r="AI224" s="3" t="n"/>
+      <c r="AJ224" s="3" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="3" t="n"/>
@@ -9137,6 +9371,7 @@
       <c r="AG225" s="3" t="n"/>
       <c r="AH225" s="3" t="n"/>
       <c r="AI225" s="3" t="n"/>
+      <c r="AJ225" s="3" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="3" t="n"/>
@@ -9174,6 +9409,7 @@
       <c r="AG226" s="3" t="n"/>
       <c r="AH226" s="3" t="n"/>
       <c r="AI226" s="3" t="n"/>
+      <c r="AJ226" s="3" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="3" t="n"/>
@@ -9211,6 +9447,7 @@
       <c r="AG227" s="3" t="n"/>
       <c r="AH227" s="3" t="n"/>
       <c r="AI227" s="3" t="n"/>
+      <c r="AJ227" s="3" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="3" t="n"/>
@@ -9248,6 +9485,7 @@
       <c r="AG228" s="3" t="n"/>
       <c r="AH228" s="3" t="n"/>
       <c r="AI228" s="3" t="n"/>
+      <c r="AJ228" s="3" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="3" t="n"/>
@@ -9285,6 +9523,7 @@
       <c r="AG229" s="3" t="n"/>
       <c r="AH229" s="3" t="n"/>
       <c r="AI229" s="3" t="n"/>
+      <c r="AJ229" s="3" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="3" t="n"/>
@@ -9322,6 +9561,7 @@
       <c r="AG230" s="3" t="n"/>
       <c r="AH230" s="3" t="n"/>
       <c r="AI230" s="3" t="n"/>
+      <c r="AJ230" s="3" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="3" t="n"/>
@@ -9359,6 +9599,7 @@
       <c r="AG231" s="3" t="n"/>
       <c r="AH231" s="3" t="n"/>
       <c r="AI231" s="3" t="n"/>
+      <c r="AJ231" s="3" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="3" t="n"/>
@@ -9396,6 +9637,7 @@
       <c r="AG232" s="3" t="n"/>
       <c r="AH232" s="3" t="n"/>
       <c r="AI232" s="3" t="n"/>
+      <c r="AJ232" s="3" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="3" t="n"/>
@@ -9433,6 +9675,7 @@
       <c r="AG233" s="3" t="n"/>
       <c r="AH233" s="3" t="n"/>
       <c r="AI233" s="3" t="n"/>
+      <c r="AJ233" s="3" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="3" t="n"/>
@@ -9470,6 +9713,7 @@
       <c r="AG234" s="3" t="n"/>
       <c r="AH234" s="3" t="n"/>
       <c r="AI234" s="3" t="n"/>
+      <c r="AJ234" s="3" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="3" t="n"/>
@@ -9507,6 +9751,7 @@
       <c r="AG235" s="3" t="n"/>
       <c r="AH235" s="3" t="n"/>
       <c r="AI235" s="3" t="n"/>
+      <c r="AJ235" s="3" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="3" t="n"/>
@@ -9544,6 +9789,7 @@
       <c r="AG236" s="3" t="n"/>
       <c r="AH236" s="3" t="n"/>
       <c r="AI236" s="3" t="n"/>
+      <c r="AJ236" s="3" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="3" t="n"/>
@@ -9581,6 +9827,7 @@
       <c r="AG237" s="3" t="n"/>
       <c r="AH237" s="3" t="n"/>
       <c r="AI237" s="3" t="n"/>
+      <c r="AJ237" s="3" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="3" t="n"/>
@@ -9618,6 +9865,7 @@
       <c r="AG238" s="3" t="n"/>
       <c r="AH238" s="3" t="n"/>
       <c r="AI238" s="3" t="n"/>
+      <c r="AJ238" s="3" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="3" t="n"/>
@@ -9655,6 +9903,7 @@
       <c r="AG239" s="3" t="n"/>
       <c r="AH239" s="3" t="n"/>
       <c r="AI239" s="3" t="n"/>
+      <c r="AJ239" s="3" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="3" t="n"/>
@@ -9692,6 +9941,7 @@
       <c r="AG240" s="3" t="n"/>
       <c r="AH240" s="3" t="n"/>
       <c r="AI240" s="3" t="n"/>
+      <c r="AJ240" s="3" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="3" t="n"/>
@@ -9729,6 +9979,7 @@
       <c r="AG241" s="3" t="n"/>
       <c r="AH241" s="3" t="n"/>
       <c r="AI241" s="3" t="n"/>
+      <c r="AJ241" s="3" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="3" t="n"/>
@@ -9766,6 +10017,7 @@
       <c r="AG242" s="3" t="n"/>
       <c r="AH242" s="3" t="n"/>
       <c r="AI242" s="3" t="n"/>
+      <c r="AJ242" s="3" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="3" t="n"/>
@@ -9803,6 +10055,7 @@
       <c r="AG243" s="3" t="n"/>
       <c r="AH243" s="3" t="n"/>
       <c r="AI243" s="3" t="n"/>
+      <c r="AJ243" s="3" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="3" t="n"/>
@@ -9840,6 +10093,7 @@
       <c r="AG244" s="3" t="n"/>
       <c r="AH244" s="3" t="n"/>
       <c r="AI244" s="3" t="n"/>
+      <c r="AJ244" s="3" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="3" t="n"/>
@@ -9877,6 +10131,7 @@
       <c r="AG245" s="3" t="n"/>
       <c r="AH245" s="3" t="n"/>
       <c r="AI245" s="3" t="n"/>
+      <c r="AJ245" s="3" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="3" t="n"/>
@@ -9914,6 +10169,7 @@
       <c r="AG246" s="3" t="n"/>
       <c r="AH246" s="3" t="n"/>
       <c r="AI246" s="3" t="n"/>
+      <c r="AJ246" s="3" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="3" t="n"/>
@@ -9951,6 +10207,7 @@
       <c r="AG247" s="3" t="n"/>
       <c r="AH247" s="3" t="n"/>
       <c r="AI247" s="3" t="n"/>
+      <c r="AJ247" s="3" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="3" t="n"/>
@@ -9988,6 +10245,7 @@
       <c r="AG248" s="3" t="n"/>
       <c r="AH248" s="3" t="n"/>
       <c r="AI248" s="3" t="n"/>
+      <c r="AJ248" s="3" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="3" t="n"/>
@@ -10025,6 +10283,7 @@
       <c r="AG249" s="3" t="n"/>
       <c r="AH249" s="3" t="n"/>
       <c r="AI249" s="3" t="n"/>
+      <c r="AJ249" s="3" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="3" t="n"/>
@@ -10062,6 +10321,7 @@
       <c r="AG250" s="3" t="n"/>
       <c r="AH250" s="3" t="n"/>
       <c r="AI250" s="3" t="n"/>
+      <c r="AJ250" s="3" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="3" t="n"/>
@@ -10099,6 +10359,7 @@
       <c r="AG251" s="3" t="n"/>
       <c r="AH251" s="3" t="n"/>
       <c r="AI251" s="3" t="n"/>
+      <c r="AJ251" s="3" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="3" t="n"/>
@@ -10136,6 +10397,7 @@
       <c r="AG252" s="3" t="n"/>
       <c r="AH252" s="3" t="n"/>
       <c r="AI252" s="3" t="n"/>
+      <c r="AJ252" s="3" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="3" t="n"/>
@@ -10173,6 +10435,7 @@
       <c r="AG253" s="3" t="n"/>
       <c r="AH253" s="3" t="n"/>
       <c r="AI253" s="3" t="n"/>
+      <c r="AJ253" s="3" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="3" t="n"/>
@@ -10210,6 +10473,7 @@
       <c r="AG254" s="3" t="n"/>
       <c r="AH254" s="3" t="n"/>
       <c r="AI254" s="3" t="n"/>
+      <c r="AJ254" s="3" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="3" t="n"/>
@@ -10247,6 +10511,7 @@
       <c r="AG255" s="3" t="n"/>
       <c r="AH255" s="3" t="n"/>
       <c r="AI255" s="3" t="n"/>
+      <c r="AJ255" s="3" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="3" t="n"/>
@@ -10284,6 +10549,7 @@
       <c r="AG256" s="3" t="n"/>
       <c r="AH256" s="3" t="n"/>
       <c r="AI256" s="3" t="n"/>
+      <c r="AJ256" s="3" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="3" t="n"/>
@@ -10321,6 +10587,7 @@
       <c r="AG257" s="3" t="n"/>
       <c r="AH257" s="3" t="n"/>
       <c r="AI257" s="3" t="n"/>
+      <c r="AJ257" s="3" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n"/>
@@ -10358,6 +10625,7 @@
       <c r="AG258" s="3" t="n"/>
       <c r="AH258" s="3" t="n"/>
       <c r="AI258" s="3" t="n"/>
+      <c r="AJ258" s="3" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="3" t="n"/>
@@ -10395,6 +10663,7 @@
       <c r="AG259" s="3" t="n"/>
       <c r="AH259" s="3" t="n"/>
       <c r="AI259" s="3" t="n"/>
+      <c r="AJ259" s="3" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="3" t="n"/>
@@ -10432,6 +10701,7 @@
       <c r="AG260" s="3" t="n"/>
       <c r="AH260" s="3" t="n"/>
       <c r="AI260" s="3" t="n"/>
+      <c r="AJ260" s="3" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="3" t="n"/>
@@ -10469,6 +10739,7 @@
       <c r="AG261" s="3" t="n"/>
       <c r="AH261" s="3" t="n"/>
       <c r="AI261" s="3" t="n"/>
+      <c r="AJ261" s="3" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="3" t="n"/>
@@ -10506,6 +10777,7 @@
       <c r="AG262" s="3" t="n"/>
       <c r="AH262" s="3" t="n"/>
       <c r="AI262" s="3" t="n"/>
+      <c r="AJ262" s="3" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="3" t="n"/>
@@ -10543,6 +10815,7 @@
       <c r="AG263" s="3" t="n"/>
       <c r="AH263" s="3" t="n"/>
       <c r="AI263" s="3" t="n"/>
+      <c r="AJ263" s="3" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="3" t="n"/>
@@ -10580,6 +10853,7 @@
       <c r="AG264" s="3" t="n"/>
       <c r="AH264" s="3" t="n"/>
       <c r="AI264" s="3" t="n"/>
+      <c r="AJ264" s="3" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="3" t="n"/>
@@ -10617,6 +10891,7 @@
       <c r="AG265" s="3" t="n"/>
       <c r="AH265" s="3" t="n"/>
       <c r="AI265" s="3" t="n"/>
+      <c r="AJ265" s="3" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="3" t="n"/>
@@ -10654,6 +10929,7 @@
       <c r="AG266" s="3" t="n"/>
       <c r="AH266" s="3" t="n"/>
       <c r="AI266" s="3" t="n"/>
+      <c r="AJ266" s="3" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="3" t="n"/>
@@ -10691,6 +10967,7 @@
       <c r="AG267" s="3" t="n"/>
       <c r="AH267" s="3" t="n"/>
       <c r="AI267" s="3" t="n"/>
+      <c r="AJ267" s="3" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="3" t="n"/>
@@ -10728,6 +11005,7 @@
       <c r="AG268" s="3" t="n"/>
       <c r="AH268" s="3" t="n"/>
       <c r="AI268" s="3" t="n"/>
+      <c r="AJ268" s="3" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="3" t="n"/>
@@ -10765,6 +11043,7 @@
       <c r="AG269" s="3" t="n"/>
       <c r="AH269" s="3" t="n"/>
       <c r="AI269" s="3" t="n"/>
+      <c r="AJ269" s="3" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="3" t="n"/>
@@ -10802,6 +11081,7 @@
       <c r="AG270" s="3" t="n"/>
       <c r="AH270" s="3" t="n"/>
       <c r="AI270" s="3" t="n"/>
+      <c r="AJ270" s="3" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="3" t="n"/>
@@ -10839,6 +11119,7 @@
       <c r="AG271" s="3" t="n"/>
       <c r="AH271" s="3" t="n"/>
       <c r="AI271" s="3" t="n"/>
+      <c r="AJ271" s="3" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="3" t="n"/>
@@ -10876,6 +11157,7 @@
       <c r="AG272" s="3" t="n"/>
       <c r="AH272" s="3" t="n"/>
       <c r="AI272" s="3" t="n"/>
+      <c r="AJ272" s="3" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="3" t="n"/>
@@ -10913,6 +11195,7 @@
       <c r="AG273" s="3" t="n"/>
       <c r="AH273" s="3" t="n"/>
       <c r="AI273" s="3" t="n"/>
+      <c r="AJ273" s="3" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="3" t="n"/>
@@ -10950,6 +11233,7 @@
       <c r="AG274" s="3" t="n"/>
       <c r="AH274" s="3" t="n"/>
       <c r="AI274" s="3" t="n"/>
+      <c r="AJ274" s="3" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="3" t="n"/>
@@ -10987,6 +11271,7 @@
       <c r="AG275" s="3" t="n"/>
       <c r="AH275" s="3" t="n"/>
       <c r="AI275" s="3" t="n"/>
+      <c r="AJ275" s="3" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="3" t="n"/>
@@ -11024,6 +11309,7 @@
       <c r="AG276" s="3" t="n"/>
       <c r="AH276" s="3" t="n"/>
       <c r="AI276" s="3" t="n"/>
+      <c r="AJ276" s="3" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="3" t="n"/>
@@ -11061,6 +11347,7 @@
       <c r="AG277" s="3" t="n"/>
       <c r="AH277" s="3" t="n"/>
       <c r="AI277" s="3" t="n"/>
+      <c r="AJ277" s="3" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="3" t="n"/>
@@ -11098,6 +11385,7 @@
       <c r="AG278" s="3" t="n"/>
       <c r="AH278" s="3" t="n"/>
       <c r="AI278" s="3" t="n"/>
+      <c r="AJ278" s="3" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="3" t="n"/>
@@ -11135,6 +11423,7 @@
       <c r="AG279" s="3" t="n"/>
       <c r="AH279" s="3" t="n"/>
       <c r="AI279" s="3" t="n"/>
+      <c r="AJ279" s="3" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="3" t="n"/>
@@ -11172,6 +11461,7 @@
       <c r="AG280" s="3" t="n"/>
       <c r="AH280" s="3" t="n"/>
       <c r="AI280" s="3" t="n"/>
+      <c r="AJ280" s="3" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="3" t="n"/>
@@ -11209,6 +11499,7 @@
       <c r="AG281" s="3" t="n"/>
       <c r="AH281" s="3" t="n"/>
       <c r="AI281" s="3" t="n"/>
+      <c r="AJ281" s="3" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="3" t="n"/>
@@ -11246,6 +11537,7 @@
       <c r="AG282" s="3" t="n"/>
       <c r="AH282" s="3" t="n"/>
       <c r="AI282" s="3" t="n"/>
+      <c r="AJ282" s="3" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="3" t="n"/>
@@ -11283,6 +11575,7 @@
       <c r="AG283" s="3" t="n"/>
       <c r="AH283" s="3" t="n"/>
       <c r="AI283" s="3" t="n"/>
+      <c r="AJ283" s="3" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="3" t="n"/>
@@ -11320,6 +11613,7 @@
       <c r="AG284" s="3" t="n"/>
       <c r="AH284" s="3" t="n"/>
       <c r="AI284" s="3" t="n"/>
+      <c r="AJ284" s="3" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="3" t="n"/>
@@ -11357,6 +11651,7 @@
       <c r="AG285" s="3" t="n"/>
       <c r="AH285" s="3" t="n"/>
       <c r="AI285" s="3" t="n"/>
+      <c r="AJ285" s="3" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="3" t="n"/>
@@ -11394,6 +11689,7 @@
       <c r="AG286" s="3" t="n"/>
       <c r="AH286" s="3" t="n"/>
       <c r="AI286" s="3" t="n"/>
+      <c r="AJ286" s="3" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="3" t="n"/>
@@ -11431,6 +11727,7 @@
       <c r="AG287" s="3" t="n"/>
       <c r="AH287" s="3" t="n"/>
       <c r="AI287" s="3" t="n"/>
+      <c r="AJ287" s="3" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="3" t="n"/>
@@ -11468,6 +11765,7 @@
       <c r="AG288" s="3" t="n"/>
       <c r="AH288" s="3" t="n"/>
       <c r="AI288" s="3" t="n"/>
+      <c r="AJ288" s="3" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="3" t="n"/>
@@ -11505,6 +11803,7 @@
       <c r="AG289" s="3" t="n"/>
       <c r="AH289" s="3" t="n"/>
       <c r="AI289" s="3" t="n"/>
+      <c r="AJ289" s="3" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="3" t="n"/>
@@ -11542,6 +11841,7 @@
       <c r="AG290" s="3" t="n"/>
       <c r="AH290" s="3" t="n"/>
       <c r="AI290" s="3" t="n"/>
+      <c r="AJ290" s="3" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="3" t="n"/>
@@ -11579,6 +11879,7 @@
       <c r="AG291" s="3" t="n"/>
       <c r="AH291" s="3" t="n"/>
       <c r="AI291" s="3" t="n"/>
+      <c r="AJ291" s="3" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="3" t="n"/>
@@ -11616,6 +11917,7 @@
       <c r="AG292" s="3" t="n"/>
       <c r="AH292" s="3" t="n"/>
       <c r="AI292" s="3" t="n"/>
+      <c r="AJ292" s="3" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="3" t="n"/>
@@ -11653,6 +11955,7 @@
       <c r="AG293" s="3" t="n"/>
       <c r="AH293" s="3" t="n"/>
       <c r="AI293" s="3" t="n"/>
+      <c r="AJ293" s="3" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="3" t="n"/>
@@ -11690,6 +11993,7 @@
       <c r="AG294" s="3" t="n"/>
       <c r="AH294" s="3" t="n"/>
       <c r="AI294" s="3" t="n"/>
+      <c r="AJ294" s="3" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="3" t="n"/>
@@ -11727,6 +12031,7 @@
       <c r="AG295" s="3" t="n"/>
       <c r="AH295" s="3" t="n"/>
       <c r="AI295" s="3" t="n"/>
+      <c r="AJ295" s="3" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="3" t="n"/>
@@ -11764,6 +12069,7 @@
       <c r="AG296" s="3" t="n"/>
       <c r="AH296" s="3" t="n"/>
       <c r="AI296" s="3" t="n"/>
+      <c r="AJ296" s="3" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="3" t="n"/>
@@ -11801,6 +12107,7 @@
       <c r="AG297" s="3" t="n"/>
       <c r="AH297" s="3" t="n"/>
       <c r="AI297" s="3" t="n"/>
+      <c r="AJ297" s="3" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="3" t="n"/>
@@ -11838,6 +12145,7 @@
       <c r="AG298" s="3" t="n"/>
       <c r="AH298" s="3" t="n"/>
       <c r="AI298" s="3" t="n"/>
+      <c r="AJ298" s="3" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="3" t="n"/>
@@ -11875,6 +12183,7 @@
       <c r="AG299" s="3" t="n"/>
       <c r="AH299" s="3" t="n"/>
       <c r="AI299" s="3" t="n"/>
+      <c r="AJ299" s="3" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="3" t="n"/>
@@ -11912,6 +12221,7 @@
       <c r="AG300" s="3" t="n"/>
       <c r="AH300" s="3" t="n"/>
       <c r="AI300" s="3" t="n"/>
+      <c r="AJ300" s="3" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="3" t="n"/>
@@ -11949,6 +12259,7 @@
       <c r="AG301" s="3" t="n"/>
       <c r="AH301" s="3" t="n"/>
       <c r="AI301" s="3" t="n"/>
+      <c r="AJ301" s="3" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="3" t="n"/>
@@ -11986,6 +12297,7 @@
       <c r="AG302" s="3" t="n"/>
       <c r="AH302" s="3" t="n"/>
       <c r="AI302" s="3" t="n"/>
+      <c r="AJ302" s="3" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="3" t="n"/>
@@ -12023,6 +12335,7 @@
       <c r="AG303" s="3" t="n"/>
       <c r="AH303" s="3" t="n"/>
       <c r="AI303" s="3" t="n"/>
+      <c r="AJ303" s="3" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="3" t="n"/>
@@ -12060,6 +12373,7 @@
       <c r="AG304" s="3" t="n"/>
       <c r="AH304" s="3" t="n"/>
       <c r="AI304" s="3" t="n"/>
+      <c r="AJ304" s="3" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="3" t="n"/>
@@ -12097,6 +12411,7 @@
       <c r="AG305" s="3" t="n"/>
       <c r="AH305" s="3" t="n"/>
       <c r="AI305" s="3" t="n"/>
+      <c r="AJ305" s="3" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="3" t="n"/>
@@ -12134,6 +12449,7 @@
       <c r="AG306" s="3" t="n"/>
       <c r="AH306" s="3" t="n"/>
       <c r="AI306" s="3" t="n"/>
+      <c r="AJ306" s="3" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="3" t="n"/>
@@ -12171,6 +12487,7 @@
       <c r="AG307" s="3" t="n"/>
       <c r="AH307" s="3" t="n"/>
       <c r="AI307" s="3" t="n"/>
+      <c r="AJ307" s="3" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="3" t="n"/>
@@ -12208,6 +12525,7 @@
       <c r="AG308" s="3" t="n"/>
       <c r="AH308" s="3" t="n"/>
       <c r="AI308" s="3" t="n"/>
+      <c r="AJ308" s="3" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="3" t="n"/>
@@ -12245,6 +12563,7 @@
       <c r="AG309" s="3" t="n"/>
       <c r="AH309" s="3" t="n"/>
       <c r="AI309" s="3" t="n"/>
+      <c r="AJ309" s="3" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="3" t="n"/>
@@ -12282,6 +12601,7 @@
       <c r="AG310" s="3" t="n"/>
       <c r="AH310" s="3" t="n"/>
       <c r="AI310" s="3" t="n"/>
+      <c r="AJ310" s="3" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="3" t="n"/>
@@ -12319,6 +12639,7 @@
       <c r="AG311" s="3" t="n"/>
       <c r="AH311" s="3" t="n"/>
       <c r="AI311" s="3" t="n"/>
+      <c r="AJ311" s="3" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="3" t="n"/>
@@ -12356,6 +12677,7 @@
       <c r="AG312" s="3" t="n"/>
       <c r="AH312" s="3" t="n"/>
       <c r="AI312" s="3" t="n"/>
+      <c r="AJ312" s="3" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="3" t="n"/>
@@ -12393,6 +12715,7 @@
       <c r="AG313" s="3" t="n"/>
       <c r="AH313" s="3" t="n"/>
       <c r="AI313" s="3" t="n"/>
+      <c r="AJ313" s="3" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="3" t="n"/>
@@ -12430,6 +12753,7 @@
       <c r="AG314" s="3" t="n"/>
       <c r="AH314" s="3" t="n"/>
       <c r="AI314" s="3" t="n"/>
+      <c r="AJ314" s="3" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="3" t="n"/>
@@ -12467,6 +12791,7 @@
       <c r="AG315" s="3" t="n"/>
       <c r="AH315" s="3" t="n"/>
       <c r="AI315" s="3" t="n"/>
+      <c r="AJ315" s="3" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="3" t="n"/>
@@ -12504,6 +12829,7 @@
       <c r="AG316" s="3" t="n"/>
       <c r="AH316" s="3" t="n"/>
       <c r="AI316" s="3" t="n"/>
+      <c r="AJ316" s="3" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="3" t="n"/>
@@ -12541,6 +12867,7 @@
       <c r="AG317" s="3" t="n"/>
       <c r="AH317" s="3" t="n"/>
       <c r="AI317" s="3" t="n"/>
+      <c r="AJ317" s="3" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="3" t="n"/>
@@ -12578,6 +12905,7 @@
       <c r="AG318" s="3" t="n"/>
       <c r="AH318" s="3" t="n"/>
       <c r="AI318" s="3" t="n"/>
+      <c r="AJ318" s="3" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="3" t="n"/>
@@ -12615,6 +12943,7 @@
       <c r="AG319" s="3" t="n"/>
       <c r="AH319" s="3" t="n"/>
       <c r="AI319" s="3" t="n"/>
+      <c r="AJ319" s="3" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="3" t="n"/>
@@ -12652,6 +12981,7 @@
       <c r="AG320" s="3" t="n"/>
       <c r="AH320" s="3" t="n"/>
       <c r="AI320" s="3" t="n"/>
+      <c r="AJ320" s="3" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="3" t="n"/>
@@ -12689,6 +13019,7 @@
       <c r="AG321" s="3" t="n"/>
       <c r="AH321" s="3" t="n"/>
       <c r="AI321" s="3" t="n"/>
+      <c r="AJ321" s="3" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="3" t="n"/>
@@ -12726,6 +13057,7 @@
       <c r="AG322" s="3" t="n"/>
       <c r="AH322" s="3" t="n"/>
       <c r="AI322" s="3" t="n"/>
+      <c r="AJ322" s="3" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="3" t="n"/>
@@ -12763,6 +13095,7 @@
       <c r="AG323" s="3" t="n"/>
       <c r="AH323" s="3" t="n"/>
       <c r="AI323" s="3" t="n"/>
+      <c r="AJ323" s="3" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="3" t="n"/>
@@ -12800,6 +13133,7 @@
       <c r="AG324" s="3" t="n"/>
       <c r="AH324" s="3" t="n"/>
       <c r="AI324" s="3" t="n"/>
+      <c r="AJ324" s="3" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="3" t="n"/>
@@ -12837,6 +13171,7 @@
       <c r="AG325" s="3" t="n"/>
       <c r="AH325" s="3" t="n"/>
       <c r="AI325" s="3" t="n"/>
+      <c r="AJ325" s="3" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="3" t="n"/>
@@ -12874,6 +13209,7 @@
       <c r="AG326" s="3" t="n"/>
       <c r="AH326" s="3" t="n"/>
       <c r="AI326" s="3" t="n"/>
+      <c r="AJ326" s="3" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="3" t="n"/>
@@ -12911,6 +13247,7 @@
       <c r="AG327" s="3" t="n"/>
       <c r="AH327" s="3" t="n"/>
       <c r="AI327" s="3" t="n"/>
+      <c r="AJ327" s="3" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="3" t="n"/>
@@ -12948,6 +13285,7 @@
       <c r="AG328" s="3" t="n"/>
       <c r="AH328" s="3" t="n"/>
       <c r="AI328" s="3" t="n"/>
+      <c r="AJ328" s="3" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="3" t="n"/>
@@ -12985,6 +13323,7 @@
       <c r="AG329" s="3" t="n"/>
       <c r="AH329" s="3" t="n"/>
       <c r="AI329" s="3" t="n"/>
+      <c r="AJ329" s="3" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="3" t="n"/>
@@ -13022,6 +13361,7 @@
       <c r="AG330" s="3" t="n"/>
       <c r="AH330" s="3" t="n"/>
       <c r="AI330" s="3" t="n"/>
+      <c r="AJ330" s="3" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="3" t="n"/>
@@ -13059,6 +13399,7 @@
       <c r="AG331" s="3" t="n"/>
       <c r="AH331" s="3" t="n"/>
       <c r="AI331" s="3" t="n"/>
+      <c r="AJ331" s="3" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="3" t="n"/>
@@ -13096,6 +13437,7 @@
       <c r="AG332" s="3" t="n"/>
       <c r="AH332" s="3" t="n"/>
       <c r="AI332" s="3" t="n"/>
+      <c r="AJ332" s="3" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="3" t="n"/>
@@ -13133,6 +13475,7 @@
       <c r="AG333" s="3" t="n"/>
       <c r="AH333" s="3" t="n"/>
       <c r="AI333" s="3" t="n"/>
+      <c r="AJ333" s="3" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="3" t="n"/>
@@ -13170,6 +13513,7 @@
       <c r="AG334" s="3" t="n"/>
       <c r="AH334" s="3" t="n"/>
       <c r="AI334" s="3" t="n"/>
+      <c r="AJ334" s="3" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="3" t="n"/>
@@ -13207,6 +13551,7 @@
       <c r="AG335" s="3" t="n"/>
       <c r="AH335" s="3" t="n"/>
       <c r="AI335" s="3" t="n"/>
+      <c r="AJ335" s="3" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="3" t="n"/>
@@ -13244,6 +13589,7 @@
       <c r="AG336" s="3" t="n"/>
       <c r="AH336" s="3" t="n"/>
       <c r="AI336" s="3" t="n"/>
+      <c r="AJ336" s="3" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="3" t="n"/>
@@ -13281,6 +13627,7 @@
       <c r="AG337" s="3" t="n"/>
       <c r="AH337" s="3" t="n"/>
       <c r="AI337" s="3" t="n"/>
+      <c r="AJ337" s="3" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="3" t="n"/>
@@ -13318,6 +13665,7 @@
       <c r="AG338" s="3" t="n"/>
       <c r="AH338" s="3" t="n"/>
       <c r="AI338" s="3" t="n"/>
+      <c r="AJ338" s="3" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="3" t="n"/>
@@ -13355,6 +13703,7 @@
       <c r="AG339" s="3" t="n"/>
       <c r="AH339" s="3" t="n"/>
       <c r="AI339" s="3" t="n"/>
+      <c r="AJ339" s="3" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="3" t="n"/>
@@ -13392,6 +13741,7 @@
       <c r="AG340" s="3" t="n"/>
       <c r="AH340" s="3" t="n"/>
       <c r="AI340" s="3" t="n"/>
+      <c r="AJ340" s="3" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="3" t="n"/>
@@ -13429,6 +13779,7 @@
       <c r="AG341" s="3" t="n"/>
       <c r="AH341" s="3" t="n"/>
       <c r="AI341" s="3" t="n"/>
+      <c r="AJ341" s="3" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="3" t="n"/>
@@ -13466,6 +13817,7 @@
       <c r="AG342" s="3" t="n"/>
       <c r="AH342" s="3" t="n"/>
       <c r="AI342" s="3" t="n"/>
+      <c r="AJ342" s="3" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="3" t="n"/>
@@ -13503,6 +13855,7 @@
       <c r="AG343" s="3" t="n"/>
       <c r="AH343" s="3" t="n"/>
       <c r="AI343" s="3" t="n"/>
+      <c r="AJ343" s="3" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="3" t="n"/>
@@ -13540,6 +13893,7 @@
       <c r="AG344" s="3" t="n"/>
       <c r="AH344" s="3" t="n"/>
       <c r="AI344" s="3" t="n"/>
+      <c r="AJ344" s="3" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="3" t="n"/>
@@ -13577,6 +13931,7 @@
       <c r="AG345" s="3" t="n"/>
       <c r="AH345" s="3" t="n"/>
       <c r="AI345" s="3" t="n"/>
+      <c r="AJ345" s="3" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="3" t="n"/>
@@ -13614,6 +13969,7 @@
       <c r="AG346" s="3" t="n"/>
       <c r="AH346" s="3" t="n"/>
       <c r="AI346" s="3" t="n"/>
+      <c r="AJ346" s="3" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="3" t="n"/>
@@ -13651,6 +14007,7 @@
       <c r="AG347" s="3" t="n"/>
       <c r="AH347" s="3" t="n"/>
       <c r="AI347" s="3" t="n"/>
+      <c r="AJ347" s="3" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="3" t="n"/>
@@ -13688,6 +14045,7 @@
       <c r="AG348" s="3" t="n"/>
       <c r="AH348" s="3" t="n"/>
       <c r="AI348" s="3" t="n"/>
+      <c r="AJ348" s="3" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="3" t="n"/>
@@ -13725,6 +14083,7 @@
       <c r="AG349" s="3" t="n"/>
       <c r="AH349" s="3" t="n"/>
       <c r="AI349" s="3" t="n"/>
+      <c r="AJ349" s="3" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="3" t="n"/>
@@ -13762,6 +14121,7 @@
       <c r="AG350" s="3" t="n"/>
       <c r="AH350" s="3" t="n"/>
       <c r="AI350" s="3" t="n"/>
+      <c r="AJ350" s="3" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="3" t="n"/>
@@ -13799,6 +14159,7 @@
       <c r="AG351" s="3" t="n"/>
       <c r="AH351" s="3" t="n"/>
       <c r="AI351" s="3" t="n"/>
+      <c r="AJ351" s="3" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="3" t="n"/>
@@ -13836,6 +14197,7 @@
       <c r="AG352" s="3" t="n"/>
       <c r="AH352" s="3" t="n"/>
       <c r="AI352" s="3" t="n"/>
+      <c r="AJ352" s="3" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="3" t="n"/>
@@ -13873,6 +14235,7 @@
       <c r="AG353" s="3" t="n"/>
       <c r="AH353" s="3" t="n"/>
       <c r="AI353" s="3" t="n"/>
+      <c r="AJ353" s="3" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="3" t="n"/>
@@ -13910,6 +14273,7 @@
       <c r="AG354" s="3" t="n"/>
       <c r="AH354" s="3" t="n"/>
       <c r="AI354" s="3" t="n"/>
+      <c r="AJ354" s="3" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="3" t="n"/>
@@ -13947,6 +14311,7 @@
       <c r="AG355" s="3" t="n"/>
       <c r="AH355" s="3" t="n"/>
       <c r="AI355" s="3" t="n"/>
+      <c r="AJ355" s="3" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="3" t="n"/>
@@ -13984,6 +14349,7 @@
       <c r="AG356" s="3" t="n"/>
       <c r="AH356" s="3" t="n"/>
       <c r="AI356" s="3" t="n"/>
+      <c r="AJ356" s="3" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="3" t="n"/>
@@ -14021,6 +14387,7 @@
       <c r="AG357" s="3" t="n"/>
       <c r="AH357" s="3" t="n"/>
       <c r="AI357" s="3" t="n"/>
+      <c r="AJ357" s="3" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="3" t="n"/>
@@ -14058,6 +14425,7 @@
       <c r="AG358" s="3" t="n"/>
       <c r="AH358" s="3" t="n"/>
       <c r="AI358" s="3" t="n"/>
+      <c r="AJ358" s="3" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="3" t="n"/>
@@ -14095,6 +14463,7 @@
       <c r="AG359" s="3" t="n"/>
       <c r="AH359" s="3" t="n"/>
       <c r="AI359" s="3" t="n"/>
+      <c r="AJ359" s="3" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="3" t="n"/>
@@ -14132,6 +14501,7 @@
       <c r="AG360" s="3" t="n"/>
       <c r="AH360" s="3" t="n"/>
       <c r="AI360" s="3" t="n"/>
+      <c r="AJ360" s="3" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="3" t="n"/>
@@ -14169,6 +14539,7 @@
       <c r="AG361" s="3" t="n"/>
       <c r="AH361" s="3" t="n"/>
       <c r="AI361" s="3" t="n"/>
+      <c r="AJ361" s="3" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="3" t="n"/>
@@ -14206,6 +14577,7 @@
       <c r="AG362" s="3" t="n"/>
       <c r="AH362" s="3" t="n"/>
       <c r="AI362" s="3" t="n"/>
+      <c r="AJ362" s="3" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="3" t="n"/>
@@ -14243,6 +14615,7 @@
       <c r="AG363" s="3" t="n"/>
       <c r="AH363" s="3" t="n"/>
       <c r="AI363" s="3" t="n"/>
+      <c r="AJ363" s="3" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="3" t="n"/>
@@ -14280,6 +14653,7 @@
       <c r="AG364" s="3" t="n"/>
       <c r="AH364" s="3" t="n"/>
       <c r="AI364" s="3" t="n"/>
+      <c r="AJ364" s="3" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="3" t="n"/>
@@ -14317,6 +14691,7 @@
       <c r="AG365" s="3" t="n"/>
       <c r="AH365" s="3" t="n"/>
       <c r="AI365" s="3" t="n"/>
+      <c r="AJ365" s="3" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="3" t="n"/>
@@ -14354,6 +14729,7 @@
       <c r="AG366" s="3" t="n"/>
       <c r="AH366" s="3" t="n"/>
       <c r="AI366" s="3" t="n"/>
+      <c r="AJ366" s="3" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="3" t="n"/>
@@ -14391,6 +14767,7 @@
       <c r="AG367" s="3" t="n"/>
       <c r="AH367" s="3" t="n"/>
       <c r="AI367" s="3" t="n"/>
+      <c r="AJ367" s="3" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="3" t="n"/>
@@ -14428,6 +14805,7 @@
       <c r="AG368" s="3" t="n"/>
       <c r="AH368" s="3" t="n"/>
       <c r="AI368" s="3" t="n"/>
+      <c r="AJ368" s="3" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="3" t="n"/>
@@ -14465,6 +14843,7 @@
       <c r="AG369" s="3" t="n"/>
       <c r="AH369" s="3" t="n"/>
       <c r="AI369" s="3" t="n"/>
+      <c r="AJ369" s="3" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="3" t="n"/>
@@ -14502,6 +14881,7 @@
       <c r="AG370" s="3" t="n"/>
       <c r="AH370" s="3" t="n"/>
       <c r="AI370" s="3" t="n"/>
+      <c r="AJ370" s="3" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="3" t="n"/>
@@ -14539,6 +14919,7 @@
       <c r="AG371" s="3" t="n"/>
       <c r="AH371" s="3" t="n"/>
       <c r="AI371" s="3" t="n"/>
+      <c r="AJ371" s="3" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="3" t="n"/>
@@ -14576,6 +14957,7 @@
       <c r="AG372" s="3" t="n"/>
       <c r="AH372" s="3" t="n"/>
       <c r="AI372" s="3" t="n"/>
+      <c r="AJ372" s="3" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="3" t="n"/>
@@ -14613,6 +14995,7 @@
       <c r="AG373" s="3" t="n"/>
       <c r="AH373" s="3" t="n"/>
       <c r="AI373" s="3" t="n"/>
+      <c r="AJ373" s="3" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="3" t="n"/>
@@ -14650,6 +15033,7 @@
       <c r="AG374" s="3" t="n"/>
       <c r="AH374" s="3" t="n"/>
       <c r="AI374" s="3" t="n"/>
+      <c r="AJ374" s="3" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="3" t="n"/>
@@ -14687,6 +15071,7 @@
       <c r="AG375" s="3" t="n"/>
       <c r="AH375" s="3" t="n"/>
       <c r="AI375" s="3" t="n"/>
+      <c r="AJ375" s="3" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="3" t="n"/>
@@ -14724,6 +15109,7 @@
       <c r="AG376" s="3" t="n"/>
       <c r="AH376" s="3" t="n"/>
       <c r="AI376" s="3" t="n"/>
+      <c r="AJ376" s="3" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="3" t="n"/>
@@ -14761,6 +15147,7 @@
       <c r="AG377" s="3" t="n"/>
       <c r="AH377" s="3" t="n"/>
       <c r="AI377" s="3" t="n"/>
+      <c r="AJ377" s="3" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="3" t="n"/>
@@ -14798,6 +15185,7 @@
       <c r="AG378" s="3" t="n"/>
       <c r="AH378" s="3" t="n"/>
       <c r="AI378" s="3" t="n"/>
+      <c r="AJ378" s="3" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="3" t="n"/>
@@ -14835,6 +15223,7 @@
       <c r="AG379" s="3" t="n"/>
       <c r="AH379" s="3" t="n"/>
       <c r="AI379" s="3" t="n"/>
+      <c r="AJ379" s="3" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="3" t="n"/>
@@ -14872,6 +15261,7 @@
       <c r="AG380" s="3" t="n"/>
       <c r="AH380" s="3" t="n"/>
       <c r="AI380" s="3" t="n"/>
+      <c r="AJ380" s="3" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="3" t="n"/>
@@ -14909,6 +15299,7 @@
       <c r="AG381" s="3" t="n"/>
       <c r="AH381" s="3" t="n"/>
       <c r="AI381" s="3" t="n"/>
+      <c r="AJ381" s="3" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="3" t="n"/>
@@ -14946,6 +15337,7 @@
       <c r="AG382" s="3" t="n"/>
       <c r="AH382" s="3" t="n"/>
       <c r="AI382" s="3" t="n"/>
+      <c r="AJ382" s="3" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="3" t="n"/>
@@ -14983,6 +15375,7 @@
       <c r="AG383" s="3" t="n"/>
       <c r="AH383" s="3" t="n"/>
       <c r="AI383" s="3" t="n"/>
+      <c r="AJ383" s="3" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="3" t="n"/>
@@ -15020,6 +15413,7 @@
       <c r="AG384" s="3" t="n"/>
       <c r="AH384" s="3" t="n"/>
       <c r="AI384" s="3" t="n"/>
+      <c r="AJ384" s="3" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="3" t="n"/>
@@ -15057,6 +15451,7 @@
       <c r="AG385" s="3" t="n"/>
       <c r="AH385" s="3" t="n"/>
       <c r="AI385" s="3" t="n"/>
+      <c r="AJ385" s="3" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="3" t="n"/>
@@ -15094,6 +15489,7 @@
       <c r="AG386" s="3" t="n"/>
       <c r="AH386" s="3" t="n"/>
       <c r="AI386" s="3" t="n"/>
+      <c r="AJ386" s="3" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="3" t="n"/>
@@ -15131,6 +15527,7 @@
       <c r="AG387" s="3" t="n"/>
       <c r="AH387" s="3" t="n"/>
       <c r="AI387" s="3" t="n"/>
+      <c r="AJ387" s="3" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="3" t="n"/>
@@ -15168,6 +15565,7 @@
       <c r="AG388" s="3" t="n"/>
       <c r="AH388" s="3" t="n"/>
       <c r="AI388" s="3" t="n"/>
+      <c r="AJ388" s="3" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="3" t="n"/>
@@ -15205,6 +15603,7 @@
       <c r="AG389" s="3" t="n"/>
       <c r="AH389" s="3" t="n"/>
       <c r="AI389" s="3" t="n"/>
+      <c r="AJ389" s="3" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="3" t="n"/>
@@ -15242,6 +15641,7 @@
       <c r="AG390" s="3" t="n"/>
       <c r="AH390" s="3" t="n"/>
       <c r="AI390" s="3" t="n"/>
+      <c r="AJ390" s="3" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="3" t="n"/>
@@ -15279,6 +15679,7 @@
       <c r="AG391" s="3" t="n"/>
       <c r="AH391" s="3" t="n"/>
       <c r="AI391" s="3" t="n"/>
+      <c r="AJ391" s="3" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="3" t="n"/>
@@ -15316,6 +15717,7 @@
       <c r="AG392" s="3" t="n"/>
       <c r="AH392" s="3" t="n"/>
       <c r="AI392" s="3" t="n"/>
+      <c r="AJ392" s="3" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="3" t="n"/>
@@ -15353,6 +15755,7 @@
       <c r="AG393" s="3" t="n"/>
       <c r="AH393" s="3" t="n"/>
       <c r="AI393" s="3" t="n"/>
+      <c r="AJ393" s="3" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="3" t="n"/>
@@ -15390,6 +15793,7 @@
       <c r="AG394" s="3" t="n"/>
       <c r="AH394" s="3" t="n"/>
       <c r="AI394" s="3" t="n"/>
+      <c r="AJ394" s="3" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="3" t="n"/>
@@ -15427,6 +15831,7 @@
       <c r="AG395" s="3" t="n"/>
       <c r="AH395" s="3" t="n"/>
       <c r="AI395" s="3" t="n"/>
+      <c r="AJ395" s="3" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="3" t="n"/>
@@ -15464,6 +15869,7 @@
       <c r="AG396" s="3" t="n"/>
       <c r="AH396" s="3" t="n"/>
       <c r="AI396" s="3" t="n"/>
+      <c r="AJ396" s="3" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="3" t="n"/>
@@ -15501,6 +15907,7 @@
       <c r="AG397" s="3" t="n"/>
       <c r="AH397" s="3" t="n"/>
       <c r="AI397" s="3" t="n"/>
+      <c r="AJ397" s="3" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="3" t="n"/>
@@ -15538,6 +15945,7 @@
       <c r="AG398" s="3" t="n"/>
       <c r="AH398" s="3" t="n"/>
       <c r="AI398" s="3" t="n"/>
+      <c r="AJ398" s="3" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="3" t="n"/>
@@ -15575,6 +15983,7 @@
       <c r="AG399" s="3" t="n"/>
       <c r="AH399" s="3" t="n"/>
       <c r="AI399" s="3" t="n"/>
+      <c r="AJ399" s="3" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="3" t="n"/>
@@ -15612,6 +16021,7 @@
       <c r="AG400" s="3" t="n"/>
       <c r="AH400" s="3" t="n"/>
       <c r="AI400" s="3" t="n"/>
+      <c r="AJ400" s="3" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="3" t="n"/>
@@ -15649,6 +16059,7 @@
       <c r="AG401" s="3" t="n"/>
       <c r="AH401" s="3" t="n"/>
       <c r="AI401" s="3" t="n"/>
+      <c r="AJ401" s="3" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="3" t="n"/>
@@ -15686,6 +16097,7 @@
       <c r="AG402" s="3" t="n"/>
       <c r="AH402" s="3" t="n"/>
       <c r="AI402" s="3" t="n"/>
+      <c r="AJ402" s="3" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="3" t="n"/>
@@ -15723,6 +16135,7 @@
       <c r="AG403" s="3" t="n"/>
       <c r="AH403" s="3" t="n"/>
       <c r="AI403" s="3" t="n"/>
+      <c r="AJ403" s="3" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="3" t="n"/>
@@ -15760,6 +16173,7 @@
       <c r="AG404" s="3" t="n"/>
       <c r="AH404" s="3" t="n"/>
       <c r="AI404" s="3" t="n"/>
+      <c r="AJ404" s="3" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="3" t="n"/>
@@ -15797,6 +16211,7 @@
       <c r="AG405" s="3" t="n"/>
       <c r="AH405" s="3" t="n"/>
       <c r="AI405" s="3" t="n"/>
+      <c r="AJ405" s="3" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="3" t="n"/>
@@ -15834,6 +16249,7 @@
       <c r="AG406" s="3" t="n"/>
       <c r="AH406" s="3" t="n"/>
       <c r="AI406" s="3" t="n"/>
+      <c r="AJ406" s="3" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="3" t="n"/>
@@ -15871,6 +16287,7 @@
       <c r="AG407" s="3" t="n"/>
       <c r="AH407" s="3" t="n"/>
       <c r="AI407" s="3" t="n"/>
+      <c r="AJ407" s="3" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="3" t="n"/>
@@ -15908,6 +16325,7 @@
       <c r="AG408" s="3" t="n"/>
       <c r="AH408" s="3" t="n"/>
       <c r="AI408" s="3" t="n"/>
+      <c r="AJ408" s="3" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="3" t="n"/>
@@ -15945,6 +16363,7 @@
       <c r="AG409" s="3" t="n"/>
       <c r="AH409" s="3" t="n"/>
       <c r="AI409" s="3" t="n"/>
+      <c r="AJ409" s="3" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="3" t="n"/>
@@ -15982,6 +16401,7 @@
       <c r="AG410" s="3" t="n"/>
       <c r="AH410" s="3" t="n"/>
       <c r="AI410" s="3" t="n"/>
+      <c r="AJ410" s="3" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="3" t="n"/>
@@ -16019,6 +16439,7 @@
       <c r="AG411" s="3" t="n"/>
       <c r="AH411" s="3" t="n"/>
       <c r="AI411" s="3" t="n"/>
+      <c r="AJ411" s="3" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="3" t="n"/>
@@ -16056,6 +16477,7 @@
       <c r="AG412" s="3" t="n"/>
       <c r="AH412" s="3" t="n"/>
       <c r="AI412" s="3" t="n"/>
+      <c r="AJ412" s="3" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="3" t="n"/>
@@ -16093,6 +16515,7 @@
       <c r="AG413" s="3" t="n"/>
       <c r="AH413" s="3" t="n"/>
       <c r="AI413" s="3" t="n"/>
+      <c r="AJ413" s="3" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="3" t="n"/>
@@ -16130,6 +16553,7 @@
       <c r="AG414" s="3" t="n"/>
       <c r="AH414" s="3" t="n"/>
       <c r="AI414" s="3" t="n"/>
+      <c r="AJ414" s="3" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="3" t="n"/>
@@ -16167,6 +16591,7 @@
       <c r="AG415" s="3" t="n"/>
       <c r="AH415" s="3" t="n"/>
       <c r="AI415" s="3" t="n"/>
+      <c r="AJ415" s="3" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="3" t="n"/>
@@ -16204,6 +16629,7 @@
       <c r="AG416" s="3" t="n"/>
       <c r="AH416" s="3" t="n"/>
       <c r="AI416" s="3" t="n"/>
+      <c r="AJ416" s="3" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="3" t="n"/>
@@ -16241,6 +16667,7 @@
       <c r="AG417" s="3" t="n"/>
       <c r="AH417" s="3" t="n"/>
       <c r="AI417" s="3" t="n"/>
+      <c r="AJ417" s="3" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="3" t="n"/>
@@ -16278,6 +16705,7 @@
       <c r="AG418" s="3" t="n"/>
       <c r="AH418" s="3" t="n"/>
       <c r="AI418" s="3" t="n"/>
+      <c r="AJ418" s="3" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="3" t="n"/>
@@ -16315,6 +16743,7 @@
       <c r="AG419" s="3" t="n"/>
       <c r="AH419" s="3" t="n"/>
       <c r="AI419" s="3" t="n"/>
+      <c r="AJ419" s="3" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="3" t="n"/>
@@ -16352,6 +16781,7 @@
       <c r="AG420" s="3" t="n"/>
       <c r="AH420" s="3" t="n"/>
       <c r="AI420" s="3" t="n"/>
+      <c r="AJ420" s="3" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="3" t="n"/>
@@ -16389,6 +16819,7 @@
       <c r="AG421" s="3" t="n"/>
       <c r="AH421" s="3" t="n"/>
       <c r="AI421" s="3" t="n"/>
+      <c r="AJ421" s="3" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="3" t="n"/>
@@ -16426,6 +16857,7 @@
       <c r="AG422" s="3" t="n"/>
       <c r="AH422" s="3" t="n"/>
       <c r="AI422" s="3" t="n"/>
+      <c r="AJ422" s="3" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="3" t="n"/>
@@ -16463,6 +16895,7 @@
       <c r="AG423" s="3" t="n"/>
       <c r="AH423" s="3" t="n"/>
       <c r="AI423" s="3" t="n"/>
+      <c r="AJ423" s="3" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="3" t="n"/>
@@ -16500,6 +16933,7 @@
       <c r="AG424" s="3" t="n"/>
       <c r="AH424" s="3" t="n"/>
       <c r="AI424" s="3" t="n"/>
+      <c r="AJ424" s="3" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="3" t="n"/>
@@ -16537,6 +16971,7 @@
       <c r="AG425" s="3" t="n"/>
       <c r="AH425" s="3" t="n"/>
       <c r="AI425" s="3" t="n"/>
+      <c r="AJ425" s="3" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="3" t="n"/>
@@ -16574,6 +17009,7 @@
       <c r="AG426" s="3" t="n"/>
       <c r="AH426" s="3" t="n"/>
       <c r="AI426" s="3" t="n"/>
+      <c r="AJ426" s="3" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="3" t="n"/>
@@ -16611,6 +17047,7 @@
       <c r="AG427" s="3" t="n"/>
       <c r="AH427" s="3" t="n"/>
       <c r="AI427" s="3" t="n"/>
+      <c r="AJ427" s="3" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="3" t="n"/>
@@ -16648,6 +17085,7 @@
       <c r="AG428" s="3" t="n"/>
       <c r="AH428" s="3" t="n"/>
       <c r="AI428" s="3" t="n"/>
+      <c r="AJ428" s="3" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="3" t="n"/>
@@ -16685,6 +17123,7 @@
       <c r="AG429" s="3" t="n"/>
       <c r="AH429" s="3" t="n"/>
       <c r="AI429" s="3" t="n"/>
+      <c r="AJ429" s="3" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="3" t="n"/>
@@ -16722,6 +17161,7 @@
       <c r="AG430" s="3" t="n"/>
       <c r="AH430" s="3" t="n"/>
       <c r="AI430" s="3" t="n"/>
+      <c r="AJ430" s="3" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="3" t="n"/>
@@ -16759,6 +17199,7 @@
       <c r="AG431" s="3" t="n"/>
       <c r="AH431" s="3" t="n"/>
       <c r="AI431" s="3" t="n"/>
+      <c r="AJ431" s="3" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="3" t="n"/>
@@ -16796,6 +17237,7 @@
       <c r="AG432" s="3" t="n"/>
       <c r="AH432" s="3" t="n"/>
       <c r="AI432" s="3" t="n"/>
+      <c r="AJ432" s="3" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="3" t="n"/>
@@ -16833,6 +17275,7 @@
       <c r="AG433" s="3" t="n"/>
       <c r="AH433" s="3" t="n"/>
       <c r="AI433" s="3" t="n"/>
+      <c r="AJ433" s="3" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="3" t="n"/>
@@ -16870,6 +17313,7 @@
       <c r="AG434" s="3" t="n"/>
       <c r="AH434" s="3" t="n"/>
       <c r="AI434" s="3" t="n"/>
+      <c r="AJ434" s="3" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="3" t="n"/>
@@ -16907,6 +17351,7 @@
       <c r="AG435" s="3" t="n"/>
       <c r="AH435" s="3" t="n"/>
       <c r="AI435" s="3" t="n"/>
+      <c r="AJ435" s="3" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="3" t="n"/>
@@ -16944,6 +17389,7 @@
       <c r="AG436" s="3" t="n"/>
       <c r="AH436" s="3" t="n"/>
       <c r="AI436" s="3" t="n"/>
+      <c r="AJ436" s="3" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="3" t="n"/>
@@ -16981,6 +17427,7 @@
       <c r="AG437" s="3" t="n"/>
       <c r="AH437" s="3" t="n"/>
       <c r="AI437" s="3" t="n"/>
+      <c r="AJ437" s="3" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="3" t="n"/>
@@ -17018,6 +17465,7 @@
       <c r="AG438" s="3" t="n"/>
       <c r="AH438" s="3" t="n"/>
       <c r="AI438" s="3" t="n"/>
+      <c r="AJ438" s="3" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="3" t="n"/>
@@ -17055,6 +17503,7 @@
       <c r="AG439" s="3" t="n"/>
       <c r="AH439" s="3" t="n"/>
       <c r="AI439" s="3" t="n"/>
+      <c r="AJ439" s="3" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="3" t="n"/>
@@ -17092,6 +17541,7 @@
       <c r="AG440" s="3" t="n"/>
       <c r="AH440" s="3" t="n"/>
       <c r="AI440" s="3" t="n"/>
+      <c r="AJ440" s="3" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="3" t="n"/>
@@ -17129,6 +17579,7 @@
       <c r="AG441" s="3" t="n"/>
       <c r="AH441" s="3" t="n"/>
       <c r="AI441" s="3" t="n"/>
+      <c r="AJ441" s="3" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="3" t="n"/>
@@ -17166,6 +17617,7 @@
       <c r="AG442" s="3" t="n"/>
       <c r="AH442" s="3" t="n"/>
       <c r="AI442" s="3" t="n"/>
+      <c r="AJ442" s="3" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="3" t="n"/>
@@ -17203,6 +17655,7 @@
       <c r="AG443" s="3" t="n"/>
       <c r="AH443" s="3" t="n"/>
       <c r="AI443" s="3" t="n"/>
+      <c r="AJ443" s="3" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="3" t="n"/>
@@ -17240,6 +17693,7 @@
       <c r="AG444" s="3" t="n"/>
       <c r="AH444" s="3" t="n"/>
       <c r="AI444" s="3" t="n"/>
+      <c r="AJ444" s="3" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="3" t="n"/>
@@ -17277,6 +17731,7 @@
       <c r="AG445" s="3" t="n"/>
       <c r="AH445" s="3" t="n"/>
       <c r="AI445" s="3" t="n"/>
+      <c r="AJ445" s="3" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="3" t="n"/>
@@ -17314,6 +17769,7 @@
       <c r="AG446" s="3" t="n"/>
       <c r="AH446" s="3" t="n"/>
       <c r="AI446" s="3" t="n"/>
+      <c r="AJ446" s="3" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="3" t="n"/>
@@ -17351,6 +17807,7 @@
       <c r="AG447" s="3" t="n"/>
       <c r="AH447" s="3" t="n"/>
       <c r="AI447" s="3" t="n"/>
+      <c r="AJ447" s="3" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="3" t="n"/>
@@ -17388,6 +17845,7 @@
       <c r="AG448" s="3" t="n"/>
       <c r="AH448" s="3" t="n"/>
       <c r="AI448" s="3" t="n"/>
+      <c r="AJ448" s="3" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="3" t="n"/>
@@ -17425,6 +17883,7 @@
       <c r="AG449" s="3" t="n"/>
       <c r="AH449" s="3" t="n"/>
       <c r="AI449" s="3" t="n"/>
+      <c r="AJ449" s="3" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="3" t="n"/>
@@ -17462,6 +17921,7 @@
       <c r="AG450" s="3" t="n"/>
       <c r="AH450" s="3" t="n"/>
       <c r="AI450" s="3" t="n"/>
+      <c r="AJ450" s="3" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="3" t="n"/>
@@ -17499,6 +17959,7 @@
       <c r="AG451" s="3" t="n"/>
       <c r="AH451" s="3" t="n"/>
       <c r="AI451" s="3" t="n"/>
+      <c r="AJ451" s="3" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="3" t="n"/>
@@ -17536,6 +17997,7 @@
       <c r="AG452" s="3" t="n"/>
       <c r="AH452" s="3" t="n"/>
       <c r="AI452" s="3" t="n"/>
+      <c r="AJ452" s="3" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="3" t="n"/>
@@ -17573,6 +18035,7 @@
       <c r="AG453" s="3" t="n"/>
       <c r="AH453" s="3" t="n"/>
       <c r="AI453" s="3" t="n"/>
+      <c r="AJ453" s="3" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="3" t="n"/>
@@ -17610,6 +18073,7 @@
       <c r="AG454" s="3" t="n"/>
       <c r="AH454" s="3" t="n"/>
       <c r="AI454" s="3" t="n"/>
+      <c r="AJ454" s="3" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="3" t="n"/>
@@ -17647,6 +18111,7 @@
       <c r="AG455" s="3" t="n"/>
       <c r="AH455" s="3" t="n"/>
       <c r="AI455" s="3" t="n"/>
+      <c r="AJ455" s="3" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="3" t="n"/>
@@ -17684,6 +18149,7 @@
       <c r="AG456" s="3" t="n"/>
       <c r="AH456" s="3" t="n"/>
       <c r="AI456" s="3" t="n"/>
+      <c r="AJ456" s="3" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="3" t="n"/>
@@ -17721,6 +18187,7 @@
       <c r="AG457" s="3" t="n"/>
       <c r="AH457" s="3" t="n"/>
       <c r="AI457" s="3" t="n"/>
+      <c r="AJ457" s="3" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="3" t="n"/>
@@ -17758,6 +18225,7 @@
       <c r="AG458" s="3" t="n"/>
       <c r="AH458" s="3" t="n"/>
       <c r="AI458" s="3" t="n"/>
+      <c r="AJ458" s="3" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="3" t="n"/>
@@ -17795,6 +18263,7 @@
       <c r="AG459" s="3" t="n"/>
       <c r="AH459" s="3" t="n"/>
       <c r="AI459" s="3" t="n"/>
+      <c r="AJ459" s="3" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="3" t="n"/>
@@ -17832,6 +18301,7 @@
       <c r="AG460" s="3" t="n"/>
       <c r="AH460" s="3" t="n"/>
       <c r="AI460" s="3" t="n"/>
+      <c r="AJ460" s="3" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="3" t="n"/>
@@ -17869,6 +18339,7 @@
       <c r="AG461" s="3" t="n"/>
       <c r="AH461" s="3" t="n"/>
       <c r="AI461" s="3" t="n"/>
+      <c r="AJ461" s="3" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="3" t="n"/>
@@ -17906,6 +18377,7 @@
       <c r="AG462" s="3" t="n"/>
       <c r="AH462" s="3" t="n"/>
       <c r="AI462" s="3" t="n"/>
+      <c r="AJ462" s="3" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="3" t="n"/>
@@ -17943,6 +18415,7 @@
       <c r="AG463" s="3" t="n"/>
       <c r="AH463" s="3" t="n"/>
       <c r="AI463" s="3" t="n"/>
+      <c r="AJ463" s="3" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="3" t="n"/>
@@ -17980,6 +18453,7 @@
       <c r="AG464" s="3" t="n"/>
       <c r="AH464" s="3" t="n"/>
       <c r="AI464" s="3" t="n"/>
+      <c r="AJ464" s="3" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="3" t="n"/>
@@ -18017,6 +18491,7 @@
       <c r="AG465" s="3" t="n"/>
       <c r="AH465" s="3" t="n"/>
       <c r="AI465" s="3" t="n"/>
+      <c r="AJ465" s="3" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="3" t="n"/>
@@ -18054,6 +18529,7 @@
       <c r="AG466" s="3" t="n"/>
       <c r="AH466" s="3" t="n"/>
       <c r="AI466" s="3" t="n"/>
+      <c r="AJ466" s="3" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="3" t="n"/>
@@ -18091,6 +18567,7 @@
       <c r="AG467" s="3" t="n"/>
       <c r="AH467" s="3" t="n"/>
       <c r="AI467" s="3" t="n"/>
+      <c r="AJ467" s="3" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="3" t="n"/>
@@ -18128,6 +18605,7 @@
       <c r="AG468" s="3" t="n"/>
       <c r="AH468" s="3" t="n"/>
       <c r="AI468" s="3" t="n"/>
+      <c r="AJ468" s="3" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="3" t="n"/>
@@ -18165,6 +18643,7 @@
       <c r="AG469" s="3" t="n"/>
       <c r="AH469" s="3" t="n"/>
       <c r="AI469" s="3" t="n"/>
+      <c r="AJ469" s="3" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="3" t="n"/>
@@ -18202,6 +18681,7 @@
       <c r="AG470" s="3" t="n"/>
       <c r="AH470" s="3" t="n"/>
       <c r="AI470" s="3" t="n"/>
+      <c r="AJ470" s="3" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="3" t="n"/>
@@ -18239,6 +18719,7 @@
       <c r="AG471" s="3" t="n"/>
       <c r="AH471" s="3" t="n"/>
       <c r="AI471" s="3" t="n"/>
+      <c r="AJ471" s="3" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="3" t="n"/>
@@ -18276,6 +18757,7 @@
       <c r="AG472" s="3" t="n"/>
       <c r="AH472" s="3" t="n"/>
       <c r="AI472" s="3" t="n"/>
+      <c r="AJ472" s="3" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="3" t="n"/>
@@ -18313,6 +18795,7 @@
       <c r="AG473" s="3" t="n"/>
       <c r="AH473" s="3" t="n"/>
       <c r="AI473" s="3" t="n"/>
+      <c r="AJ473" s="3" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="3" t="n"/>
@@ -18350,6 +18833,7 @@
       <c r="AG474" s="3" t="n"/>
       <c r="AH474" s="3" t="n"/>
       <c r="AI474" s="3" t="n"/>
+      <c r="AJ474" s="3" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="3" t="n"/>
@@ -18387,6 +18871,7 @@
       <c r="AG475" s="3" t="n"/>
       <c r="AH475" s="3" t="n"/>
       <c r="AI475" s="3" t="n"/>
+      <c r="AJ475" s="3" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="3" t="n"/>
@@ -18424,6 +18909,7 @@
       <c r="AG476" s="3" t="n"/>
       <c r="AH476" s="3" t="n"/>
       <c r="AI476" s="3" t="n"/>
+      <c r="AJ476" s="3" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="3" t="n"/>
@@ -18461,6 +18947,7 @@
       <c r="AG477" s="3" t="n"/>
       <c r="AH477" s="3" t="n"/>
       <c r="AI477" s="3" t="n"/>
+      <c r="AJ477" s="3" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="3" t="n"/>
@@ -18498,6 +18985,7 @@
       <c r="AG478" s="3" t="n"/>
       <c r="AH478" s="3" t="n"/>
       <c r="AI478" s="3" t="n"/>
+      <c r="AJ478" s="3" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="3" t="n"/>
@@ -18535,6 +19023,7 @@
       <c r="AG479" s="3" t="n"/>
       <c r="AH479" s="3" t="n"/>
       <c r="AI479" s="3" t="n"/>
+      <c r="AJ479" s="3" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="3" t="n"/>
@@ -18572,6 +19061,7 @@
       <c r="AG480" s="3" t="n"/>
       <c r="AH480" s="3" t="n"/>
       <c r="AI480" s="3" t="n"/>
+      <c r="AJ480" s="3" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="3" t="n"/>
@@ -18609,6 +19099,7 @@
       <c r="AG481" s="3" t="n"/>
       <c r="AH481" s="3" t="n"/>
       <c r="AI481" s="3" t="n"/>
+      <c r="AJ481" s="3" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="3" t="n"/>
@@ -18646,6 +19137,7 @@
       <c r="AG482" s="3" t="n"/>
       <c r="AH482" s="3" t="n"/>
       <c r="AI482" s="3" t="n"/>
+      <c r="AJ482" s="3" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="3" t="n"/>
@@ -18683,6 +19175,7 @@
       <c r="AG483" s="3" t="n"/>
       <c r="AH483" s="3" t="n"/>
       <c r="AI483" s="3" t="n"/>
+      <c r="AJ483" s="3" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="3" t="n"/>
@@ -18720,6 +19213,7 @@
       <c r="AG484" s="3" t="n"/>
       <c r="AH484" s="3" t="n"/>
       <c r="AI484" s="3" t="n"/>
+      <c r="AJ484" s="3" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="3" t="n"/>
@@ -18757,6 +19251,7 @@
       <c r="AG485" s="3" t="n"/>
       <c r="AH485" s="3" t="n"/>
       <c r="AI485" s="3" t="n"/>
+      <c r="AJ485" s="3" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="3" t="n"/>
@@ -18794,6 +19289,7 @@
       <c r="AG486" s="3" t="n"/>
       <c r="AH486" s="3" t="n"/>
       <c r="AI486" s="3" t="n"/>
+      <c r="AJ486" s="3" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="3" t="n"/>
@@ -18831,6 +19327,7 @@
       <c r="AG487" s="3" t="n"/>
       <c r="AH487" s="3" t="n"/>
       <c r="AI487" s="3" t="n"/>
+      <c r="AJ487" s="3" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="3" t="n"/>
@@ -18868,6 +19365,7 @@
       <c r="AG488" s="3" t="n"/>
       <c r="AH488" s="3" t="n"/>
       <c r="AI488" s="3" t="n"/>
+      <c r="AJ488" s="3" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="3" t="n"/>
@@ -18905,6 +19403,7 @@
       <c r="AG489" s="3" t="n"/>
       <c r="AH489" s="3" t="n"/>
       <c r="AI489" s="3" t="n"/>
+      <c r="AJ489" s="3" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="3" t="n"/>
@@ -18942,6 +19441,7 @@
       <c r="AG490" s="3" t="n"/>
       <c r="AH490" s="3" t="n"/>
       <c r="AI490" s="3" t="n"/>
+      <c r="AJ490" s="3" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="3" t="n"/>
@@ -18979,6 +19479,7 @@
       <c r="AG491" s="3" t="n"/>
       <c r="AH491" s="3" t="n"/>
       <c r="AI491" s="3" t="n"/>
+      <c r="AJ491" s="3" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="3" t="n"/>
@@ -19016,6 +19517,7 @@
       <c r="AG492" s="3" t="n"/>
       <c r="AH492" s="3" t="n"/>
       <c r="AI492" s="3" t="n"/>
+      <c r="AJ492" s="3" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="3" t="n"/>
@@ -19053,6 +19555,7 @@
       <c r="AG493" s="3" t="n"/>
       <c r="AH493" s="3" t="n"/>
       <c r="AI493" s="3" t="n"/>
+      <c r="AJ493" s="3" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="3" t="n"/>
@@ -19090,6 +19593,7 @@
       <c r="AG494" s="3" t="n"/>
       <c r="AH494" s="3" t="n"/>
       <c r="AI494" s="3" t="n"/>
+      <c r="AJ494" s="3" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="3" t="n"/>
@@ -19127,6 +19631,7 @@
       <c r="AG495" s="3" t="n"/>
       <c r="AH495" s="3" t="n"/>
       <c r="AI495" s="3" t="n"/>
+      <c r="AJ495" s="3" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="3" t="n"/>
@@ -19164,6 +19669,7 @@
       <c r="AG496" s="3" t="n"/>
       <c r="AH496" s="3" t="n"/>
       <c r="AI496" s="3" t="n"/>
+      <c r="AJ496" s="3" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="3" t="n"/>
@@ -19201,6 +19707,7 @@
       <c r="AG497" s="3" t="n"/>
       <c r="AH497" s="3" t="n"/>
       <c r="AI497" s="3" t="n"/>
+      <c r="AJ497" s="3" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="3" t="n"/>
@@ -19238,6 +19745,7 @@
       <c r="AG498" s="3" t="n"/>
       <c r="AH498" s="3" t="n"/>
       <c r="AI498" s="3" t="n"/>
+      <c r="AJ498" s="3" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="3" t="n"/>
@@ -19275,6 +19783,7 @@
       <c r="AG499" s="3" t="n"/>
       <c r="AH499" s="3" t="n"/>
       <c r="AI499" s="3" t="n"/>
+      <c r="AJ499" s="3" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="3" t="n"/>
@@ -19312,6 +19821,7 @@
       <c r="AG500" s="3" t="n"/>
       <c r="AH500" s="3" t="n"/>
       <c r="AI500" s="3" t="n"/>
+      <c r="AJ500" s="3" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="3" t="n"/>
@@ -19349,9 +19859,10 @@
       <c r="AG501" s="3" t="n"/>
       <c r="AH501" s="3" t="n"/>
       <c r="AI501" s="3" t="n"/>
+      <c r="AJ501" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI501"/>
+  <autoFilter ref="A1:AJ501"/>
   <dataValidations count="5">
     <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Choose a listed value" error="Use the dropdown choices." type="list">
       <formula1>"Medical Full,Medical Task,Vocational Full,Vocational Task,Employer,Other Services"</formula1>
@@ -19380,7 +19891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -19389,7 +19900,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Unity desktop workbook — 35 operator fields; no sample patient data.</t>
+          <t>Unity desktop workbook — 36 operator fields; no sample patient data.</t>
         </is>
       </c>
     </row>
@@ -19410,40 +19921,61 @@
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>Scenario 2 All/Assign also requires NCM full name and claimant first/last names. The scenario selection is not stored in Excel. Older 35-column workbooks load NCM blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
           <t>Other values are optional. Incomplete rows load with warnings for editing.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Special instructions: up to 32,767 characters; line breaks and surrounding whitespace preserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>All other fields: up to 1,000 characters. Longer supplied values must be corrected before running.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Dates MM/DD/YYYY; time 08:30 AM. ZIPs, phones and identifiers are text. No formulas.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Blank serviceType derives Medical Full (Medical Task for Auto / Continental Tire / MI jurisdiction).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Claim jurisdiction is separate optional context entered in the app; never inferred from claimant State.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Template has no derived columns. Review defaults and jurisdiction before live work.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Loading a row never starts the portal. Select a stage and run explicitly.</t>
         </is>

</xml_diff>